<commit_message>
adding fixed #27 run
</commit_message>
<xml_diff>
--- a/aux/burgers-ch-lbm-June2026/paper_cases_table.xlsx
+++ b/aux/burgers-ch-lbm-June2026/paper_cases_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/agallojr/proj/src/q8020/q8020-cfd-experiments/aux/burgers-ch-lbm-June2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\223107543\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7395F807-0D78-8449-B3F5-5A5B2C4C0BDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4D48C5-83BF-4601-BD17-1B2BF8ACB839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3020" yWindow="1840" windowWidth="26780" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paper cases" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="125">
   <si>
     <t>#</t>
   </si>
@@ -402,6 +402,12 @@
   </si>
   <si>
     <t>steps</t>
+  </si>
+  <si>
+    <t>Rerun of above run</t>
+  </si>
+  <si>
+    <t>burgers-ch-lbm/ch_q8_c0/2026-08-28/_2c04f665/89d9be42</t>
   </si>
 </sst>
 </file>
@@ -411,7 +417,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1041,41 +1047,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE43"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:AE44"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.1640625" style="8" customWidth="1"/>
-    <col min="2" max="2" width="39.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" style="8" customWidth="1"/>
+    <col min="1" max="1" width="4.19921875" style="8" customWidth="1"/>
+    <col min="2" max="2" width="39.296875" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.296875" style="8" customWidth="1"/>
     <col min="4" max="4" width="24" style="8" customWidth="1"/>
-    <col min="5" max="5" width="4.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="4.69921875" style="8" customWidth="1"/>
     <col min="6" max="6" width="9" style="8" customWidth="1"/>
     <col min="7" max="7" width="7" style="8" customWidth="1"/>
-    <col min="8" max="9" width="5.6640625" style="8" customWidth="1"/>
+    <col min="8" max="9" width="5.69921875" style="8" customWidth="1"/>
     <col min="10" max="10" width="9.5" style="30" customWidth="1"/>
     <col min="11" max="11" width="11.5" style="21" customWidth="1"/>
     <col min="12" max="12" width="9" style="8" customWidth="1"/>
-    <col min="13" max="13" width="9.33203125" style="8" customWidth="1"/>
+    <col min="13" max="13" width="9.296875" style="8" customWidth="1"/>
     <col min="14" max="14" width="12" style="8" customWidth="1"/>
-    <col min="15" max="15" width="9.6640625" style="8" customWidth="1"/>
-    <col min="16" max="16" width="10.6640625" style="30" customWidth="1"/>
-    <col min="17" max="17" width="11.1640625" style="30" customWidth="1"/>
-    <col min="18" max="18" width="18.83203125" style="96" customWidth="1"/>
+    <col min="15" max="15" width="9.69921875" style="8" customWidth="1"/>
+    <col min="16" max="16" width="10.69921875" style="30" customWidth="1"/>
+    <col min="17" max="17" width="11.19921875" style="30" customWidth="1"/>
+    <col min="18" max="18" width="18.796875" style="96" customWidth="1"/>
     <col min="19" max="19" width="18.5" style="97" customWidth="1"/>
-    <col min="20" max="20" width="10.1640625" style="13" customWidth="1"/>
-    <col min="21" max="21" width="11.83203125" style="13" customWidth="1"/>
+    <col min="20" max="20" width="10.19921875" style="13" customWidth="1"/>
+    <col min="21" max="21" width="11.796875" style="13" customWidth="1"/>
     <col min="22" max="23" width="11.5" style="13" customWidth="1"/>
-    <col min="24" max="24" width="13.1640625" style="8" customWidth="1"/>
+    <col min="24" max="24" width="13.19921875" style="8" customWidth="1"/>
     <col min="25" max="25" width="10.5" style="77" customWidth="1"/>
-    <col min="26" max="28" width="10.83203125" style="8" customWidth="1"/>
-    <col min="29" max="29" width="11.1640625" style="8" customWidth="1"/>
-    <col min="30" max="30" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="26" max="28" width="10.796875" style="8" customWidth="1"/>
+    <col min="29" max="29" width="11.19921875" style="8" customWidth="1"/>
+    <col min="30" max="30" width="19.296875" style="8" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="89.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.83203125" style="8" customWidth="1"/>
-    <col min="33" max="16384" width="10.83203125" style="8"/>
+    <col min="32" max="32" width="10.796875" style="8" customWidth="1"/>
+    <col min="33" max="16384" width="10.796875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="9" customFormat="1" ht="17" customHeight="1">
+    <row r="1" spans="1:31" s="9" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1170,7 +1176,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:31" s="49" customFormat="1">
+    <row r="2" spans="1:31" s="49" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B2" s="49" t="s">
         <v>30</v>
       </c>
@@ -1191,7 +1197,7 @@
       <c r="S2" s="80"/>
       <c r="AE2" s="63"/>
     </row>
-    <row r="3" spans="1:31" s="1" customFormat="1">
+    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1282,7 +1288,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:31" s="1" customFormat="1">
+    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -1373,7 +1379,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="1" customFormat="1">
+    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -1464,7 +1470,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:31" s="1" customFormat="1" ht="17" customHeight="1">
+    <row r="6" spans="1:31" s="1" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -1558,7 +1564,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:31" s="1" customFormat="1">
+    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1649,7 +1655,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:31" s="1" customFormat="1">
+    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -1740,7 +1746,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="52" customFormat="1" ht="17" customHeight="1">
+    <row r="9" spans="1:31" s="52" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="52" t="s">
         <v>51</v>
       </c>
@@ -1755,7 +1761,7 @@
       </c>
       <c r="AE9" s="65"/>
     </row>
-    <row r="10" spans="1:31" s="2" customFormat="1">
+    <row r="10" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>7</v>
       </c>
@@ -1846,7 +1852,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="2" customFormat="1">
+    <row r="11" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>8</v>
       </c>
@@ -1937,7 +1943,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:31" s="2" customFormat="1">
+    <row r="12" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>9</v>
       </c>
@@ -2028,7 +2034,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:31" s="2" customFormat="1">
+    <row r="13" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>10</v>
       </c>
@@ -2119,7 +2125,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:31" s="2" customFormat="1">
+    <row r="14" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>11</v>
       </c>
@@ -2210,7 +2216,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="2" customFormat="1">
+    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>12</v>
       </c>
@@ -2301,7 +2307,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:31" s="55" customFormat="1">
+    <row r="16" spans="1:31" s="55" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B16" s="55" t="s">
         <v>63</v>
       </c>
@@ -2313,7 +2319,7 @@
       <c r="S16" s="84"/>
       <c r="AE16" s="67"/>
     </row>
-    <row r="17" spans="1:31" s="3" customFormat="1">
+    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>13</v>
       </c>
@@ -2404,7 +2410,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:31" s="3" customFormat="1">
+    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>14</v>
       </c>
@@ -2495,7 +2501,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:31" s="3" customFormat="1">
+    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>15</v>
       </c>
@@ -2586,7 +2592,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:31" s="3" customFormat="1">
+    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>16</v>
       </c>
@@ -2677,7 +2683,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:31" s="3" customFormat="1">
+    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>17</v>
       </c>
@@ -2768,7 +2774,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="1:31" s="3" customFormat="1">
+    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>18</v>
       </c>
@@ -2859,7 +2865,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="23" spans="1:31" s="46" customFormat="1" ht="17" customHeight="1">
+    <row r="23" spans="1:31" s="46" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="46" t="s">
         <v>74</v>
       </c>
@@ -2872,7 +2878,7 @@
       <c r="AD23" s="4"/>
       <c r="AE23" s="69"/>
     </row>
-    <row r="24" spans="1:31" s="4" customFormat="1" ht="17" customHeight="1">
+    <row r="24" spans="1:31" s="4" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>19</v>
       </c>
@@ -2959,7 +2965,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="25" spans="1:31" s="4" customFormat="1">
+    <row r="25" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
         <v>20</v>
       </c>
@@ -3046,7 +3052,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="1:31" s="4" customFormat="1">
+    <row r="26" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>21</v>
       </c>
@@ -3133,7 +3139,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="27" spans="1:31" s="4" customFormat="1">
+    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>22</v>
       </c>
@@ -3220,7 +3226,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="28" spans="1:31" s="4" customFormat="1">
+    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>23</v>
       </c>
@@ -3311,7 +3317,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="1:31" s="4" customFormat="1">
+    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
         <v>24</v>
       </c>
@@ -3390,7 +3396,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="30" spans="1:31" s="43" customFormat="1">
+    <row r="30" spans="1:31" s="43" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B30" s="43" t="s">
         <v>92</v>
       </c>
@@ -3402,7 +3408,7 @@
       <c r="S30" s="88"/>
       <c r="AE30" s="71"/>
     </row>
-    <row r="31" spans="1:31" s="5" customFormat="1" ht="17" customHeight="1">
+    <row r="31" spans="1:31" s="5" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5">
         <v>26</v>
       </c>
@@ -3484,10 +3490,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="1:31" s="5" customFormat="1" ht="17" customHeight="1">
-      <c r="A32" s="5">
-        <v>27</v>
-      </c>
+    <row r="32" spans="1:31" s="5" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="10" t="s">
         <v>98</v>
       </c>
@@ -3558,118 +3561,118 @@
         <v>100</v>
       </c>
     </row>
-    <row r="33" spans="1:31" s="35" customFormat="1">
-      <c r="B33" s="36" t="s">
+    <row r="33" spans="1:31" s="5" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="5">
+        <v>27</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" s="5">
+        <v>8</v>
+      </c>
+      <c r="F33" s="5">
+        <v>0.03</v>
+      </c>
+      <c r="G33" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="H33" s="5">
+        <v>0.1</v>
+      </c>
+      <c r="I33" s="5">
+        <f>N33*O33</f>
+        <v>512</v>
+      </c>
+      <c r="J33" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="K33" s="18">
+        <v>131072</v>
+      </c>
+      <c r="L33" s="5">
+        <v>4</v>
+      </c>
+      <c r="M33" s="5">
+        <v>8</v>
+      </c>
+      <c r="N33" s="5">
+        <v>512</v>
+      </c>
+      <c r="O33" s="5">
+        <v>1</v>
+      </c>
+      <c r="P33" s="27"/>
+      <c r="Q33" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="R33" s="90">
+        <v>1.0512000000000001E-2</v>
+      </c>
+      <c r="S33" s="90">
+        <v>6.3073000000000004E-2</v>
+      </c>
+      <c r="T33" s="32">
+        <v>11</v>
+      </c>
+      <c r="U33" s="32">
+        <v>15833</v>
+      </c>
+      <c r="V33" s="32">
+        <v>22033</v>
+      </c>
+      <c r="W33" s="32">
+        <v>7846</v>
+      </c>
+      <c r="X33" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y33" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z33" s="5">
+        <v>15.43</v>
+      </c>
+      <c r="AA33" s="5">
+        <v>7.19</v>
+      </c>
+      <c r="AB33" s="5">
+        <v>51.65</v>
+      </c>
+      <c r="AC33" s="5">
+        <v>349.83</v>
+      </c>
+      <c r="AD33" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE33" s="100" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="J33" s="37"/>
-      <c r="K33" s="38"/>
-      <c r="P33" s="37"/>
-      <c r="Q33" s="37"/>
-      <c r="R33" s="91"/>
-      <c r="S33" s="92"/>
-      <c r="AE33" s="73"/>
+      <c r="J34" s="37"/>
+      <c r="K34" s="38"/>
+      <c r="P34" s="37"/>
+      <c r="Q34" s="37"/>
+      <c r="R34" s="91"/>
+      <c r="S34" s="92"/>
+      <c r="AE34" s="73"/>
     </row>
-    <row r="34" spans="1:31" s="6" customFormat="1" ht="17" customHeight="1">
-      <c r="A34" s="6">
+    <row r="35" spans="1:31" s="6" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="6">
         <v>28</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B35" s="11" t="s">
         <v>102</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="E34" s="6">
-        <v>8</v>
-      </c>
-      <c r="F34" s="6">
-        <v>0.03</v>
-      </c>
-      <c r="G34" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="H34" s="6">
-        <v>0.1</v>
-      </c>
-      <c r="I34" s="6">
-        <f>N34*O34</f>
-        <v>512</v>
-      </c>
-      <c r="J34" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="K34" s="19">
-        <v>131072</v>
-      </c>
-      <c r="L34" s="6">
-        <v>4</v>
-      </c>
-      <c r="M34" s="6">
-        <v>8</v>
-      </c>
-      <c r="N34" s="6">
-        <v>2</v>
-      </c>
-      <c r="O34" s="6">
-        <v>256</v>
-      </c>
-      <c r="P34" s="28"/>
-      <c r="Q34" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="R34" s="93">
-        <v>133.57000600000001</v>
-      </c>
-      <c r="S34" s="93">
-        <v>801.40128300000003</v>
-      </c>
-      <c r="T34" s="6">
-        <v>12</v>
-      </c>
-      <c r="U34" s="6">
-        <v>31558</v>
-      </c>
-      <c r="V34" s="6">
-        <v>43515</v>
-      </c>
-      <c r="W34" s="6">
-        <v>15559</v>
-      </c>
-      <c r="X34" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y34" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="Z34" s="6">
-        <v>93.11</v>
-      </c>
-      <c r="AA34" s="6">
-        <v>54.54</v>
-      </c>
-      <c r="AB34" s="6">
-        <v>220.62</v>
-      </c>
-      <c r="AC34" s="6">
-        <v>801.33</v>
-      </c>
-      <c r="AD34" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="AE34" s="74" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="35" spans="1:31" s="6" customFormat="1" ht="17" customHeight="1">
-      <c r="A35" s="6">
-        <v>29</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>105</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>32</v>
@@ -3690,7 +3693,7 @@
         <v>0.1</v>
       </c>
       <c r="I35" s="6">
-        <f t="shared" ref="I35:I37" si="4">N35*O35</f>
+        <f>N35*O35</f>
         <v>512</v>
       </c>
       <c r="J35" s="28" t="s">
@@ -3706,32 +3709,32 @@
         <v>8</v>
       </c>
       <c r="N35" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O35" s="6">
-        <v>128</v>
+        <v>256</v>
       </c>
       <c r="P35" s="28"/>
       <c r="Q35" s="28" t="s">
         <v>95</v>
       </c>
       <c r="R35" s="93">
-        <v>82.246827999999994</v>
+        <v>133.57000600000001</v>
       </c>
       <c r="S35" s="93">
-        <v>493.469424</v>
+        <v>801.40128300000003</v>
       </c>
       <c r="T35" s="6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="U35" s="6">
-        <v>62580</v>
+        <v>31558</v>
       </c>
       <c r="V35" s="6">
-        <v>86021</v>
+        <v>43515</v>
       </c>
       <c r="W35" s="6">
-        <v>30987</v>
+        <v>15559</v>
       </c>
       <c r="X35" s="6" t="s">
         <v>42</v>
@@ -3740,30 +3743,30 @@
         <v>43</v>
       </c>
       <c r="Z35" s="6">
-        <v>170.98</v>
+        <v>93.11</v>
       </c>
       <c r="AA35" s="6">
-        <v>88.45</v>
+        <v>54.54</v>
       </c>
       <c r="AB35" s="6">
-        <v>809.67</v>
+        <v>220.62</v>
       </c>
       <c r="AC35" s="6">
-        <v>1125.3900000000001</v>
+        <v>801.33</v>
       </c>
       <c r="AD35" s="6" t="s">
         <v>47</v>
       </c>
       <c r="AE35" s="74" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
-    <row r="36" spans="1:31" s="6" customFormat="1" ht="17" customHeight="1">
+    <row r="36" spans="1:31" s="6" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="6">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>32</v>
@@ -3784,7 +3787,7 @@
         <v>0.1</v>
       </c>
       <c r="I36" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I36:I38" si="4">N36*O36</f>
         <v>512</v>
       </c>
       <c r="J36" s="28" t="s">
@@ -3800,32 +3803,32 @@
         <v>8</v>
       </c>
       <c r="N36" s="6">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O36" s="6">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="P36" s="28"/>
       <c r="Q36" s="28" t="s">
         <v>95</v>
       </c>
       <c r="R36" s="93">
-        <v>0.18355199999999999</v>
+        <v>82.246827999999994</v>
       </c>
       <c r="S36" s="93">
-        <v>1.1012850000000001</v>
+        <v>493.469424</v>
       </c>
       <c r="T36" s="6">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="U36" s="6">
-        <v>124624</v>
+        <v>62580</v>
       </c>
       <c r="V36" s="6">
-        <v>171033</v>
+        <v>86021</v>
       </c>
       <c r="W36" s="6">
-        <v>61843</v>
+        <v>30987</v>
       </c>
       <c r="X36" s="6" t="s">
         <v>42</v>
@@ -3834,30 +3837,30 @@
         <v>43</v>
       </c>
       <c r="Z36" s="6">
-        <v>107.53</v>
+        <v>170.98</v>
       </c>
       <c r="AA36" s="6">
-        <v>46.79</v>
+        <v>88.45</v>
       </c>
       <c r="AB36" s="6">
-        <v>4045.27</v>
+        <v>809.67</v>
       </c>
       <c r="AC36" s="6">
-        <v>4239.91</v>
+        <v>1125.3900000000001</v>
       </c>
       <c r="AD36" s="6" t="s">
         <v>47</v>
       </c>
       <c r="AE36" s="74" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
-    <row r="37" spans="1:31" s="6" customFormat="1" ht="17" customHeight="1">
+    <row r="37" spans="1:31" s="6" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>32</v>
@@ -3894,32 +3897,32 @@
         <v>8</v>
       </c>
       <c r="N37" s="6">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="O37" s="6">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="P37" s="28"/>
       <c r="Q37" s="28" t="s">
         <v>95</v>
       </c>
       <c r="R37" s="93">
-        <v>7.4400999999999995E-2</v>
+        <v>0.18355199999999999</v>
       </c>
       <c r="S37" s="93">
-        <v>0.44639699999999999</v>
+        <v>1.1012850000000001</v>
       </c>
       <c r="T37" s="6">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="U37" s="6">
-        <v>248712</v>
+        <v>124624</v>
       </c>
       <c r="V37" s="6">
-        <v>341057</v>
+        <v>171033</v>
       </c>
       <c r="W37" s="6">
-        <v>123555</v>
+        <v>61843</v>
       </c>
       <c r="X37" s="6" t="s">
         <v>42</v>
@@ -3928,136 +3931,136 @@
         <v>43</v>
       </c>
       <c r="Z37" s="6">
-        <v>70.45</v>
+        <v>107.53</v>
       </c>
       <c r="AA37" s="6">
-        <v>38.729999999999997</v>
+        <v>46.79</v>
       </c>
       <c r="AB37" s="6">
-        <v>92685.09</v>
+        <v>4045.27</v>
       </c>
       <c r="AC37" s="6">
-        <v>92827.3</v>
+        <v>4239.91</v>
       </c>
       <c r="AD37" s="6" t="s">
         <v>47</v>
       </c>
       <c r="AE37" s="74" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="38" spans="1:31" s="6" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="6">
+        <v>31</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="E38" s="6">
+        <v>8</v>
+      </c>
+      <c r="F38" s="6">
+        <v>0.03</v>
+      </c>
+      <c r="G38" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="H38" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="I38" s="6">
+        <f t="shared" si="4"/>
+        <v>512</v>
+      </c>
+      <c r="J38" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="K38" s="19">
+        <v>131072</v>
+      </c>
+      <c r="L38" s="6">
+        <v>4</v>
+      </c>
+      <c r="M38" s="6">
+        <v>8</v>
+      </c>
+      <c r="N38" s="6">
+        <v>16</v>
+      </c>
+      <c r="O38" s="6">
+        <v>32</v>
+      </c>
+      <c r="P38" s="28"/>
+      <c r="Q38" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="R38" s="93">
+        <v>7.4400999999999995E-2</v>
+      </c>
+      <c r="S38" s="93">
+        <v>0.44639699999999999</v>
+      </c>
+      <c r="T38" s="6">
+        <v>26</v>
+      </c>
+      <c r="U38" s="6">
+        <v>248712</v>
+      </c>
+      <c r="V38" s="6">
+        <v>341057</v>
+      </c>
+      <c r="W38" s="6">
+        <v>123555</v>
+      </c>
+      <c r="X38" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y38" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z38" s="6">
+        <v>70.45</v>
+      </c>
+      <c r="AA38" s="6">
+        <v>38.729999999999997</v>
+      </c>
+      <c r="AB38" s="6">
+        <v>92685.09</v>
+      </c>
+      <c r="AC38" s="6">
+        <v>92827.3</v>
+      </c>
+      <c r="AD38" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="AE38" s="74" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="38" spans="1:31" s="39" customFormat="1">
-      <c r="B38" s="40" t="s">
+    <row r="39" spans="1:31" s="39" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="40" t="s">
         <v>111</v>
       </c>
-      <c r="J38" s="41"/>
-      <c r="K38" s="42"/>
-      <c r="P38" s="41"/>
-      <c r="Q38" s="41"/>
-      <c r="R38" s="94"/>
-      <c r="S38" s="94"/>
-      <c r="AE38" s="75"/>
+      <c r="J39" s="41"/>
+      <c r="K39" s="42"/>
+      <c r="P39" s="41"/>
+      <c r="Q39" s="41"/>
+      <c r="R39" s="94"/>
+      <c r="S39" s="94"/>
+      <c r="AE39" s="75"/>
     </row>
-    <row r="39" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
-      <c r="A39" s="7">
+    <row r="40" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="7">
         <v>32</v>
       </c>
-      <c r="B39" s="12" t="s">
+      <c r="B40" s="12" t="s">
         <v>112</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E39" s="7">
-        <v>8</v>
-      </c>
-      <c r="F39" s="7">
-        <v>0.03</v>
-      </c>
-      <c r="G39" s="7">
-        <v>0.3</v>
-      </c>
-      <c r="H39" s="7">
-        <v>0.1</v>
-      </c>
-      <c r="I39" s="7">
-        <f>N39*O39</f>
-        <v>512</v>
-      </c>
-      <c r="J39" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="K39" s="20">
-        <v>16384</v>
-      </c>
-      <c r="L39" s="7">
-        <v>4</v>
-      </c>
-      <c r="M39" s="7">
-        <v>8</v>
-      </c>
-      <c r="N39" s="7">
-        <v>8</v>
-      </c>
-      <c r="O39" s="7">
-        <v>64</v>
-      </c>
-      <c r="P39" s="29"/>
-      <c r="Q39" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="R39" s="95">
-        <v>60.881906999999998</v>
-      </c>
-      <c r="S39" s="95">
-        <v>365.28289699999999</v>
-      </c>
-      <c r="T39" s="7">
-        <v>18</v>
-      </c>
-      <c r="U39" s="7">
-        <v>124624</v>
-      </c>
-      <c r="V39" s="7">
-        <v>171033</v>
-      </c>
-      <c r="W39" s="7">
-        <v>61843</v>
-      </c>
-      <c r="X39" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y39" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="Z39" s="7">
-        <v>298.57</v>
-      </c>
-      <c r="AA39" s="7">
-        <v>118.76</v>
-      </c>
-      <c r="AB39" s="7">
-        <v>12746.61</v>
-      </c>
-      <c r="AC39" s="7">
-        <v>13247.65</v>
-      </c>
-      <c r="AD39" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="AE39" s="76" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="40" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
-      <c r="A40" s="7">
-        <v>33</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>114</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>32</v>
@@ -4078,14 +4081,14 @@
         <v>0.1</v>
       </c>
       <c r="I40" s="7">
-        <f t="shared" ref="I40:I43" si="5">N40*O40</f>
+        <f>N40*O40</f>
         <v>512</v>
       </c>
       <c r="J40" s="29" t="s">
         <v>34</v>
       </c>
       <c r="K40" s="20">
-        <v>65536</v>
+        <v>16384</v>
       </c>
       <c r="L40" s="7">
         <v>4</v>
@@ -4104,10 +4107,10 @@
         <v>95</v>
       </c>
       <c r="R40" s="95">
-        <v>0.199902</v>
+        <v>60.881906999999998</v>
       </c>
       <c r="S40" s="95">
-        <v>1.1993819999999999</v>
+        <v>365.28289699999999</v>
       </c>
       <c r="T40" s="7">
         <v>18</v>
@@ -4128,30 +4131,30 @@
         <v>43</v>
       </c>
       <c r="Z40" s="7">
-        <v>243.68</v>
+        <v>298.57</v>
       </c>
       <c r="AA40" s="7">
-        <v>96.16</v>
+        <v>118.76</v>
       </c>
       <c r="AB40" s="7">
-        <v>12833.56</v>
+        <v>12746.61</v>
       </c>
       <c r="AC40" s="7">
-        <v>13257.85</v>
+        <v>13247.65</v>
       </c>
       <c r="AD40" s="7" t="s">
         <v>47</v>
       </c>
       <c r="AE40" s="76" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
-    <row r="41" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
+    <row r="41" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="7">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C41" s="7" t="s">
         <v>32</v>
@@ -4172,14 +4175,14 @@
         <v>0.1</v>
       </c>
       <c r="I41" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I41:I44" si="5">N41*O41</f>
         <v>512</v>
       </c>
       <c r="J41" s="29" t="s">
         <v>34</v>
       </c>
       <c r="K41" s="20">
-        <v>131072</v>
+        <v>65536</v>
       </c>
       <c r="L41" s="7">
         <v>4</v>
@@ -4198,10 +4201,10 @@
         <v>95</v>
       </c>
       <c r="R41" s="95">
-        <v>0.18355199999999999</v>
+        <v>0.199902</v>
       </c>
       <c r="S41" s="95">
-        <v>1.1012850000000001</v>
+        <v>1.1993819999999999</v>
       </c>
       <c r="T41" s="7">
         <v>18</v>
@@ -4222,30 +4225,30 @@
         <v>43</v>
       </c>
       <c r="Z41" s="7">
-        <v>285.98</v>
+        <v>243.68</v>
       </c>
       <c r="AA41" s="7">
-        <v>119.43</v>
+        <v>96.16</v>
       </c>
       <c r="AB41" s="7">
-        <v>12762.77</v>
+        <v>12833.56</v>
       </c>
       <c r="AC41" s="7">
-        <v>13257.83</v>
+        <v>13257.85</v>
       </c>
       <c r="AD41" s="7" t="s">
         <v>47</v>
       </c>
       <c r="AE41" s="76" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
-    <row r="42" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
+    <row r="42" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="7">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C42" s="7" t="s">
         <v>32</v>
@@ -4273,7 +4276,7 @@
         <v>34</v>
       </c>
       <c r="K42" s="20">
-        <v>524288</v>
+        <v>131072</v>
       </c>
       <c r="L42" s="7">
         <v>4</v>
@@ -4292,10 +4295,10 @@
         <v>95</v>
       </c>
       <c r="R42" s="95">
-        <v>8.6906999999999998E-2</v>
+        <v>0.18355199999999999</v>
       </c>
       <c r="S42" s="95">
-        <v>0.52142999999999995</v>
+        <v>1.1012850000000001</v>
       </c>
       <c r="T42" s="7">
         <v>18</v>
@@ -4316,30 +4319,30 @@
         <v>43</v>
       </c>
       <c r="Z42" s="7">
-        <v>358.19</v>
+        <v>285.98</v>
       </c>
       <c r="AA42" s="7">
-        <v>145.19999999999999</v>
+        <v>119.43</v>
       </c>
       <c r="AB42" s="7">
-        <v>12616.34</v>
+        <v>12762.77</v>
       </c>
       <c r="AC42" s="7">
-        <v>13218.02</v>
+        <v>13257.83</v>
       </c>
       <c r="AD42" s="7" t="s">
         <v>47</v>
       </c>
       <c r="AE42" s="76" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
-    <row r="43" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
+    <row r="43" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="7">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C43" s="7" t="s">
         <v>32</v>
@@ -4367,7 +4370,7 @@
         <v>34</v>
       </c>
       <c r="K43" s="20">
-        <v>1048576</v>
+        <v>524288</v>
       </c>
       <c r="L43" s="7">
         <v>4</v>
@@ -4386,10 +4389,10 @@
         <v>95</v>
       </c>
       <c r="R43" s="95">
-        <v>4.7698999999999998E-2</v>
+        <v>8.6906999999999998E-2</v>
       </c>
       <c r="S43" s="95">
-        <v>0.286186</v>
+        <v>0.52142999999999995</v>
       </c>
       <c r="T43" s="7">
         <v>18</v>
@@ -4410,21 +4413,115 @@
         <v>43</v>
       </c>
       <c r="Z43" s="7">
-        <v>274.97000000000003</v>
+        <v>358.19</v>
       </c>
       <c r="AA43" s="7">
-        <v>118.92</v>
+        <v>145.19999999999999</v>
       </c>
       <c r="AB43" s="7">
-        <v>12772.73</v>
+        <v>12616.34</v>
       </c>
       <c r="AC43" s="7">
-        <v>13259.02</v>
+        <v>13218.02</v>
       </c>
       <c r="AD43" s="7" t="s">
         <v>47</v>
       </c>
       <c r="AE43" s="76" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="44" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="7">
+        <v>36</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E44" s="7">
+        <v>8</v>
+      </c>
+      <c r="F44" s="7">
+        <v>0.03</v>
+      </c>
+      <c r="G44" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="H44" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="I44" s="7">
+        <f t="shared" si="5"/>
+        <v>512</v>
+      </c>
+      <c r="J44" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="K44" s="20">
+        <v>1048576</v>
+      </c>
+      <c r="L44" s="7">
+        <v>4</v>
+      </c>
+      <c r="M44" s="7">
+        <v>8</v>
+      </c>
+      <c r="N44" s="7">
+        <v>8</v>
+      </c>
+      <c r="O44" s="7">
+        <v>64</v>
+      </c>
+      <c r="P44" s="29"/>
+      <c r="Q44" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="R44" s="95">
+        <v>4.7698999999999998E-2</v>
+      </c>
+      <c r="S44" s="95">
+        <v>0.286186</v>
+      </c>
+      <c r="T44" s="7">
+        <v>18</v>
+      </c>
+      <c r="U44" s="7">
+        <v>124624</v>
+      </c>
+      <c r="V44" s="7">
+        <v>171033</v>
+      </c>
+      <c r="W44" s="7">
+        <v>61843</v>
+      </c>
+      <c r="X44" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y44" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z44" s="7">
+        <v>274.97000000000003</v>
+      </c>
+      <c r="AA44" s="7">
+        <v>118.92</v>
+      </c>
+      <c r="AB44" s="7">
+        <v>12772.73</v>
+      </c>
+      <c r="AC44" s="7">
+        <v>13259.02</v>
+      </c>
+      <c r="AD44" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AE44" s="76" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update paper cases table
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aux/burgers-ch-lbm-June2026/paper_cases_table.xlsx
+++ b/aux/burgers-ch-lbm-June2026/paper_cases_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\223107543\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/agallojr/proj/src/q8020/q8020-cfd-experiments/aux/burgers-ch-lbm-June2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4D48C5-83BF-4601-BD17-1B2BF8ACB839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E08B60-A77B-0D43-9253-33E799437F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19220" yWindow="2480" windowWidth="28320" windowHeight="24280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paper cases" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="121">
   <si>
     <t>#</t>
   </si>
@@ -59,9 +59,6 @@
     <t>cfl</t>
   </si>
   <si>
-    <t>Shock %</t>
-  </si>
-  <si>
     <t>Shots</t>
   </si>
   <si>
@@ -137,9 +134,6 @@
     <t>IBM Aer sim</t>
   </si>
   <si>
-    <t>~30%</t>
-  </si>
-  <si>
     <t>Fig. 1</t>
   </si>
   <si>
@@ -194,9 +188,6 @@
     <t>ab-q4/burgers_ab_show_q4_qlbm_margin.toml</t>
   </si>
   <si>
-    <t>~50%</t>
-  </si>
-  <si>
     <t>Sec IV</t>
   </si>
   <si>
@@ -230,9 +221,6 @@
     <t>ab-q4/burgers_ab_shock_q4.toml</t>
   </si>
   <si>
-    <t>~90%</t>
-  </si>
-  <si>
     <t>burgers-ch-lbm-June2026/local-mac/q4/burgers_ab_shock_q4/7ec8cce4</t>
   </si>
   <si>
@@ -266,9 +254,6 @@
     <t>ibm_kingston (Heron R2)</t>
   </si>
   <si>
-    <t>~6%</t>
-  </si>
-  <si>
     <t>TREX+DD</t>
   </si>
   <si>
@@ -408,6 +393,9 @@
   </si>
   <si>
     <t>burgers-ch-lbm/ch_q8_c0/2026-08-28/_2c04f665/89d9be42</t>
+  </si>
+  <si>
+    <t>Re</t>
   </si>
 </sst>
 </file>
@@ -417,7 +405,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1048,40 +1036,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AE44"/>
-  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="4.19921875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="39.296875" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.296875" style="8" customWidth="1"/>
+    <col min="1" max="1" width="4.1640625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="39.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" style="8" customWidth="1"/>
     <col min="4" max="4" width="24" style="8" customWidth="1"/>
-    <col min="5" max="5" width="4.69921875" style="8" customWidth="1"/>
+    <col min="5" max="5" width="4.6640625" style="8" customWidth="1"/>
     <col min="6" max="6" width="9" style="8" customWidth="1"/>
     <col min="7" max="7" width="7" style="8" customWidth="1"/>
-    <col min="8" max="9" width="5.69921875" style="8" customWidth="1"/>
-    <col min="10" max="10" width="9.5" style="30" customWidth="1"/>
+    <col min="8" max="10" width="5.6640625" style="8" customWidth="1"/>
     <col min="11" max="11" width="11.5" style="21" customWidth="1"/>
     <col min="12" max="12" width="9" style="8" customWidth="1"/>
-    <col min="13" max="13" width="9.296875" style="8" customWidth="1"/>
+    <col min="13" max="13" width="9.33203125" style="8" customWidth="1"/>
     <col min="14" max="14" width="12" style="8" customWidth="1"/>
-    <col min="15" max="15" width="9.69921875" style="8" customWidth="1"/>
-    <col min="16" max="16" width="10.69921875" style="30" customWidth="1"/>
-    <col min="17" max="17" width="11.19921875" style="30" customWidth="1"/>
-    <col min="18" max="18" width="18.796875" style="96" customWidth="1"/>
+    <col min="15" max="15" width="9.6640625" style="8" customWidth="1"/>
+    <col min="16" max="16" width="10.6640625" style="30" customWidth="1"/>
+    <col min="17" max="17" width="11.1640625" style="30" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" style="96" customWidth="1"/>
     <col min="19" max="19" width="18.5" style="97" customWidth="1"/>
-    <col min="20" max="20" width="10.19921875" style="13" customWidth="1"/>
-    <col min="21" max="21" width="11.796875" style="13" customWidth="1"/>
+    <col min="20" max="20" width="10.1640625" style="13" customWidth="1"/>
+    <col min="21" max="21" width="11.83203125" style="13" customWidth="1"/>
     <col min="22" max="23" width="11.5" style="13" customWidth="1"/>
-    <col min="24" max="24" width="13.19921875" style="8" customWidth="1"/>
+    <col min="24" max="24" width="13.1640625" style="8" customWidth="1"/>
     <col min="25" max="25" width="10.5" style="77" customWidth="1"/>
-    <col min="26" max="28" width="10.796875" style="8" customWidth="1"/>
-    <col min="29" max="29" width="11.19921875" style="8" customWidth="1"/>
-    <col min="30" max="30" width="19.296875" style="8" bestFit="1" customWidth="1"/>
+    <col min="26" max="28" width="10.83203125" style="8" customWidth="1"/>
+    <col min="29" max="29" width="11.1640625" style="8" customWidth="1"/>
+    <col min="30" max="30" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="89.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.796875" style="8" customWidth="1"/>
-    <col min="33" max="16384" width="10.796875" style="8"/>
+    <col min="32" max="32" width="10.83203125" style="8" customWidth="1"/>
+    <col min="33" max="16384" width="10.83203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="9" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" s="9" customFormat="1" ht="17" customHeight="1">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1107,78 +1094,78 @@
         <v>7</v>
       </c>
       <c r="I1" s="22" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="J1" s="22" t="s">
-        <v>8</v>
+        <v>120</v>
       </c>
       <c r="K1" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="33" t="s">
+      <c r="M1" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="33" t="s">
+      <c r="N1" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="34" t="s">
+      <c r="O1" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="34" t="s">
+      <c r="P1" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="22" t="s">
+      <c r="Q1" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="22" t="s">
+      <c r="R1" s="98" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="98" t="s">
+      <c r="S1" s="99" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="99" t="s">
+      <c r="T1" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="22" t="s">
+      <c r="U1" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="22" t="s">
+      <c r="V1" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="22" t="s">
+      <c r="W1" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="22" t="s">
+      <c r="X1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="Y1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="Z1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="AA1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="9" t="s">
+      <c r="AB1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="9" t="s">
+      <c r="AC1" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="9" t="s">
+      <c r="AD1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AE1" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="62" t="s">
+    </row>
+    <row r="2" spans="1:31" s="49" customFormat="1">
+      <c r="B2" s="49" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" s="49" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="49" t="s">
-        <v>30</v>
       </c>
       <c r="E2" s="50"/>
       <c r="F2" s="50"/>
@@ -1197,18 +1184,18 @@
       <c r="S2" s="80"/>
       <c r="AE2" s="63"/>
     </row>
-    <row r="3" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" s="1" customFormat="1">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="E3" s="1">
         <v>4</v>
@@ -1226,8 +1213,9 @@
         <f>N3*O3</f>
         <v>30</v>
       </c>
-      <c r="J3" s="23" t="s">
-        <v>34</v>
+      <c r="J3" s="1">
+        <f>G3/F3</f>
+        <v>10</v>
       </c>
       <c r="K3" s="14">
         <v>150000</v>
@@ -1246,7 +1234,7 @@
       </c>
       <c r="P3" s="23"/>
       <c r="Q3" s="23" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R3" s="81">
         <v>1.9723999999999998E-2</v>
@@ -1267,10 +1255,10 @@
         <v>1006</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y3" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z3" s="1">
         <v>0.03</v>
@@ -1285,21 +1273,21 @@
         <v>126.25</v>
       </c>
       <c r="AE3" s="64" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" s="1" customFormat="1">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="E4" s="1">
         <v>6</v>
@@ -1317,8 +1305,9 @@
         <f t="shared" ref="I4:I8" si="0">N4*O4</f>
         <v>100</v>
       </c>
-      <c r="J4" s="23" t="s">
-        <v>34</v>
+      <c r="J4" s="1">
+        <f t="shared" ref="J4:J8" si="1">G4/F4</f>
+        <v>10</v>
       </c>
       <c r="K4" s="14">
         <v>150000</v>
@@ -1337,7 +1326,7 @@
       </c>
       <c r="P4" s="23"/>
       <c r="Q4" s="23" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R4" s="81">
         <v>5.1276000000000002E-2</v>
@@ -1358,10 +1347,10 @@
         <v>6628</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y4" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z4" s="1">
         <v>0.63</v>
@@ -1376,21 +1365,21 @@
         <v>9.0399999999999991</v>
       </c>
       <c r="AE4" s="64" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" s="1" customFormat="1">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="E5" s="1">
         <v>8</v>
@@ -1408,8 +1397,9 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="J5" s="23" t="s">
-        <v>34</v>
+      <c r="J5" s="1">
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
       <c r="K5" s="14">
         <v>150000</v>
@@ -1428,7 +1418,7 @@
       </c>
       <c r="P5" s="23"/>
       <c r="Q5" s="23" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R5" s="81">
         <v>0.28409899999999999</v>
@@ -1449,10 +1439,10 @@
         <v>40272</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z5" s="1">
         <v>23.46</v>
@@ -1467,21 +1457,21 @@
         <v>182.7</v>
       </c>
       <c r="AE5" s="64" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:31" s="1" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" s="1" customFormat="1" ht="17" customHeight="1">
       <c r="A6" s="1">
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" s="1">
         <v>4</v>
@@ -1499,17 +1489,18 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="J6" s="23" t="s">
-        <v>34</v>
+      <c r="J6" s="1">
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
       <c r="K6" s="14">
         <v>150000</v>
       </c>
       <c r="L6" s="60" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M6" s="60" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N6" s="1">
         <v>1</v>
@@ -1519,7 +1510,7 @@
       </c>
       <c r="P6" s="23"/>
       <c r="Q6" s="23" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R6" s="81">
         <v>0.10970000000000001</v>
@@ -1540,10 +1531,10 @@
         <v>119440</v>
       </c>
       <c r="X6" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y6" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z6" s="1">
         <v>0.13</v>
@@ -1558,24 +1549,24 @@
         <v>9.2799999999999994</v>
       </c>
       <c r="AD6" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE6" s="64" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" s="1" customFormat="1">
       <c r="A7" s="1">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" s="1">
         <v>6</v>
@@ -1593,17 +1584,18 @@
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="J7" s="23" t="s">
-        <v>34</v>
+      <c r="J7" s="1">
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
       <c r="K7" s="14">
         <v>150000</v>
       </c>
       <c r="L7" s="60" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M7" s="60" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N7" s="1">
         <v>1</v>
@@ -1613,7 +1605,7 @@
       </c>
       <c r="P7" s="23"/>
       <c r="Q7" s="23" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R7" s="81">
         <v>1.7159000000000001E-2</v>
@@ -1634,10 +1626,10 @@
         <v>119440</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y7" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z7" s="1">
         <v>1.67</v>
@@ -1652,21 +1644,21 @@
         <v>62.72</v>
       </c>
       <c r="AE7" s="64" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" s="1" customFormat="1">
       <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E8" s="1">
         <v>8</v>
@@ -1684,17 +1676,18 @@
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="J8" s="23" t="s">
-        <v>34</v>
+      <c r="J8" s="1">
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
       <c r="K8" s="14">
         <v>150000</v>
       </c>
       <c r="L8" s="60" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M8" s="60" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N8" s="1">
         <v>1</v>
@@ -1704,7 +1697,7 @@
       </c>
       <c r="P8" s="23"/>
       <c r="Q8" s="23" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="R8" s="81">
         <v>5.7592999999999998E-2</v>
@@ -1725,10 +1718,10 @@
         <v>119440</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z8" s="1">
         <v>37.35</v>
@@ -1743,36 +1736,35 @@
         <v>1707.83</v>
       </c>
       <c r="AE8" s="64" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="52" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" s="52" customFormat="1" ht="17" customHeight="1">
       <c r="B9" s="52" t="s">
-        <v>51</v>
-      </c>
-      <c r="J9" s="53"/>
+        <v>49</v>
+      </c>
       <c r="K9" s="54"/>
       <c r="P9" s="53"/>
       <c r="Q9" s="53"/>
       <c r="R9" s="82"/>
       <c r="S9" s="82"/>
       <c r="AD9" s="78" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE9" s="65"/>
     </row>
-    <row r="10" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" s="2" customFormat="1">
       <c r="A10" s="2">
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="E10" s="2">
         <v>4</v>
@@ -1790,8 +1782,9 @@
         <f>N10*O10</f>
         <v>30</v>
       </c>
-      <c r="J10" s="24" t="s">
-        <v>53</v>
+      <c r="J10" s="2">
+        <f>G10/F10</f>
+        <v>20</v>
       </c>
       <c r="K10" s="15">
         <v>150000</v>
@@ -1810,7 +1803,7 @@
       </c>
       <c r="P10" s="24"/>
       <c r="Q10" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R10" s="83">
         <v>2.5604999999999999E-2</v>
@@ -1831,10 +1824,10 @@
         <v>1007</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y10" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z10" s="2">
         <v>0.03</v>
@@ -1849,21 +1842,21 @@
         <v>140.02000000000001</v>
       </c>
       <c r="AE10" s="66" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" s="2" customFormat="1">
       <c r="A11" s="2">
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="E11" s="2">
         <v>6</v>
@@ -1878,11 +1871,12 @@
         <v>0.1</v>
       </c>
       <c r="I11" s="2">
-        <f t="shared" ref="I11:I15" si="1">N11*O11</f>
+        <f t="shared" ref="I11:I15" si="2">N11*O11</f>
         <v>100</v>
       </c>
-      <c r="J11" s="24" t="s">
-        <v>53</v>
+      <c r="J11" s="2">
+        <f t="shared" ref="J11:J15" si="3">G11/F11</f>
+        <v>20</v>
       </c>
       <c r="K11" s="15">
         <v>150000</v>
@@ -1901,7 +1895,7 @@
       </c>
       <c r="P11" s="24"/>
       <c r="Q11" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R11" s="83">
         <v>3.783054582066233E-2</v>
@@ -1922,10 +1916,10 @@
         <v>6629</v>
       </c>
       <c r="X11" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y11" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z11" s="2">
         <v>0.61</v>
@@ -1940,21 +1934,21 @@
         <v>8.76</v>
       </c>
       <c r="AE11" s="66" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" s="2" customFormat="1">
       <c r="A12" s="2">
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="E12" s="2">
         <v>8</v>
@@ -1969,11 +1963,12 @@
         <v>0.1</v>
       </c>
       <c r="I12" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>400</v>
       </c>
-      <c r="J12" s="24" t="s">
-        <v>53</v>
+      <c r="J12" s="2">
+        <f t="shared" si="3"/>
+        <v>20</v>
       </c>
       <c r="K12" s="15">
         <v>150000</v>
@@ -1992,7 +1987,7 @@
       </c>
       <c r="P12" s="24"/>
       <c r="Q12" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R12" s="83">
         <v>84.583827999999997</v>
@@ -2013,10 +2008,10 @@
         <v>40272</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y12" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z12" s="2">
         <v>18.29</v>
@@ -2031,21 +2026,21 @@
         <v>182.51</v>
       </c>
       <c r="AE12" s="66" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" s="2" customFormat="1">
       <c r="A13" s="2">
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E13" s="2">
         <v>4</v>
@@ -2060,20 +2055,21 @@
         <v>0.1</v>
       </c>
       <c r="I13" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
-      <c r="J13" s="24" t="s">
-        <v>53</v>
+      <c r="J13" s="2">
+        <f t="shared" si="3"/>
+        <v>20</v>
       </c>
       <c r="K13" s="15">
         <v>150000</v>
       </c>
       <c r="L13" s="59" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M13" s="59" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N13" s="2">
         <v>1</v>
@@ -2083,7 +2079,7 @@
       </c>
       <c r="P13" s="24"/>
       <c r="Q13" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R13" s="83">
         <v>0.212141</v>
@@ -2104,10 +2100,10 @@
         <v>119440</v>
       </c>
       <c r="X13" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y13" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z13" s="2">
         <v>0.13</v>
@@ -2122,21 +2118,21 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="AE13" s="66" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" s="2" customFormat="1">
       <c r="A14" s="2">
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14" s="2">
         <v>6</v>
@@ -2151,20 +2147,21 @@
         <v>0.1</v>
       </c>
       <c r="I14" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>100</v>
       </c>
-      <c r="J14" s="24" t="s">
-        <v>53</v>
+      <c r="J14" s="2">
+        <f t="shared" si="3"/>
+        <v>20</v>
       </c>
       <c r="K14" s="15">
         <v>150000</v>
       </c>
       <c r="L14" s="59" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M14" s="59" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N14" s="2">
         <v>1</v>
@@ -2174,7 +2171,7 @@
       </c>
       <c r="P14" s="24"/>
       <c r="Q14" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R14" s="83">
         <v>0.100355</v>
@@ -2195,10 +2192,10 @@
         <v>119440</v>
       </c>
       <c r="X14" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y14" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z14" s="2">
         <v>1.71</v>
@@ -2213,21 +2210,21 @@
         <v>62.24</v>
       </c>
       <c r="AE14" s="66" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" s="2" customFormat="1">
       <c r="A15" s="2">
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E15" s="2">
         <v>8</v>
@@ -2242,20 +2239,21 @@
         <v>0.1</v>
       </c>
       <c r="I15" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>400</v>
       </c>
-      <c r="J15" s="24" t="s">
-        <v>53</v>
+      <c r="J15" s="2">
+        <f t="shared" si="3"/>
+        <v>20</v>
       </c>
       <c r="K15" s="15">
         <v>150000</v>
       </c>
       <c r="L15" s="59" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M15" s="59" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N15" s="2">
         <v>1</v>
@@ -2265,7 +2263,7 @@
       </c>
       <c r="P15" s="24"/>
       <c r="Q15" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R15" s="83">
         <v>7.0691000000000004E-2</v>
@@ -2286,10 +2284,10 @@
         <v>119440</v>
       </c>
       <c r="X15" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y15" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z15" s="2">
         <v>45.56</v>
@@ -2304,14 +2302,13 @@
         <v>1721.64</v>
       </c>
       <c r="AE15" s="66" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:31" s="55" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" s="55" customFormat="1">
       <c r="B16" s="55" t="s">
-        <v>63</v>
-      </c>
-      <c r="J16" s="56"/>
+        <v>60</v>
+      </c>
       <c r="K16" s="57"/>
       <c r="P16" s="56"/>
       <c r="Q16" s="56"/>
@@ -2319,18 +2316,18 @@
       <c r="S16" s="84"/>
       <c r="AE16" s="67"/>
     </row>
-    <row r="17" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" s="3" customFormat="1">
       <c r="A17" s="3">
         <v>13</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="E17" s="3">
         <v>4</v>
@@ -2348,8 +2345,9 @@
         <f>N17*O17</f>
         <v>60</v>
       </c>
-      <c r="J17" s="25" t="s">
-        <v>65</v>
+      <c r="J17" s="3">
+        <f>G17/F17</f>
+        <v>13.333333333333334</v>
       </c>
       <c r="K17" s="16">
         <v>150000</v>
@@ -2368,7 +2366,7 @@
       </c>
       <c r="P17" s="25"/>
       <c r="Q17" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R17" s="85">
         <v>1.7648E-2</v>
@@ -2389,10 +2387,10 @@
         <v>1007</v>
       </c>
       <c r="X17" s="61" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y17" s="61" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z17" s="61">
         <v>0.05</v>
@@ -2407,21 +2405,21 @@
         <v>259.93</v>
       </c>
       <c r="AE17" s="68" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" s="3" customFormat="1">
       <c r="A18" s="3">
         <v>14</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="E18" s="3">
         <v>6</v>
@@ -2436,11 +2434,12 @@
         <v>0.1</v>
       </c>
       <c r="I18" s="3">
-        <f t="shared" ref="I18:I22" si="2">N18*O18</f>
+        <f t="shared" ref="I18:I22" si="4">N18*O18</f>
         <v>230</v>
       </c>
-      <c r="J18" s="25" t="s">
-        <v>65</v>
+      <c r="J18" s="3">
+        <f t="shared" ref="J18:J22" si="5">G18/F18</f>
+        <v>13.333333333333334</v>
       </c>
       <c r="K18" s="16">
         <v>150000</v>
@@ -2459,7 +2458,7 @@
       </c>
       <c r="P18" s="25"/>
       <c r="Q18" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R18" s="85">
         <v>7.7662799853614947E-2</v>
@@ -2480,10 +2479,10 @@
         <v>6628</v>
       </c>
       <c r="X18" s="61" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y18" s="61" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z18" s="61">
         <v>1.49</v>
@@ -2498,21 +2497,21 @@
         <v>17.190000000000001</v>
       </c>
       <c r="AE18" s="68" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" s="3" customFormat="1">
       <c r="A19" s="3">
         <v>15</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="E19" s="3">
         <v>8</v>
@@ -2527,11 +2526,12 @@
         <v>0.1</v>
       </c>
       <c r="I19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>920</v>
       </c>
-      <c r="J19" s="25" t="s">
-        <v>65</v>
+      <c r="J19" s="3">
+        <f t="shared" si="5"/>
+        <v>13.333333333333334</v>
       </c>
       <c r="K19" s="16">
         <v>150000</v>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="P19" s="25"/>
       <c r="Q19" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R19" s="85">
         <v>120.614592</v>
@@ -2571,10 +2571,10 @@
         <v>40270</v>
       </c>
       <c r="X19" s="61" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y19" s="61" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z19" s="61">
         <v>55.81</v>
@@ -2589,21 +2589,21 @@
         <v>1072.96</v>
       </c>
       <c r="AE19" s="68" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" s="3" customFormat="1">
       <c r="A20" s="3">
         <v>16</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" s="3">
         <v>4</v>
@@ -2618,20 +2618,21 @@
         <v>0.1</v>
       </c>
       <c r="I20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>60</v>
       </c>
-      <c r="J20" s="25" t="s">
-        <v>65</v>
+      <c r="J20" s="3">
+        <f t="shared" si="5"/>
+        <v>13.333333333333334</v>
       </c>
       <c r="K20" s="16">
         <v>150000</v>
       </c>
       <c r="L20" s="58" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M20" s="58" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N20" s="3">
         <v>1</v>
@@ -2641,7 +2642,7 @@
       </c>
       <c r="P20" s="25"/>
       <c r="Q20" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R20" s="85">
         <v>0.15390300000000001</v>
@@ -2662,10 +2663,10 @@
         <v>119440</v>
       </c>
       <c r="X20" s="61" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y20" s="61" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z20" s="61">
         <v>0.26</v>
@@ -2680,21 +2681,21 @@
         <v>15.01</v>
       </c>
       <c r="AE20" s="68" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
-    <row r="21" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:31" s="3" customFormat="1">
       <c r="A21" s="3">
         <v>17</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E21" s="3">
         <v>6</v>
@@ -2709,20 +2710,21 @@
         <v>0.1</v>
       </c>
       <c r="I21" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>230</v>
       </c>
-      <c r="J21" s="25" t="s">
-        <v>65</v>
+      <c r="J21" s="3">
+        <f t="shared" si="5"/>
+        <v>13.333333333333334</v>
       </c>
       <c r="K21" s="16">
         <v>150000</v>
       </c>
       <c r="L21" s="58" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M21" s="58" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N21" s="3">
         <v>1</v>
@@ -2732,7 +2734,7 @@
       </c>
       <c r="P21" s="25"/>
       <c r="Q21" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R21" s="85">
         <v>4.9915000000000001E-2</v>
@@ -2753,10 +2755,10 @@
         <v>119440</v>
       </c>
       <c r="X21" s="61" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y21" s="61" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z21" s="61">
         <v>3.8</v>
@@ -2771,21 +2773,21 @@
         <v>135.74</v>
       </c>
       <c r="AE21" s="68" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
-    <row r="22" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:31" s="3" customFormat="1">
       <c r="A22" s="3">
         <v>18</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E22" s="3">
         <v>8</v>
@@ -2800,20 +2802,21 @@
         <v>0.1</v>
       </c>
       <c r="I22" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>920</v>
       </c>
-      <c r="J22" s="25" t="s">
-        <v>65</v>
+      <c r="J22" s="3">
+        <f t="shared" si="5"/>
+        <v>13.333333333333334</v>
       </c>
       <c r="K22" s="16">
         <v>150000</v>
       </c>
       <c r="L22" s="58" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M22" s="58" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="N22" s="3">
         <v>1</v>
@@ -2823,7 +2826,7 @@
       </c>
       <c r="P22" s="25"/>
       <c r="Q22" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="R22" s="85">
         <v>8.0782999999999994E-2</v>
@@ -2844,10 +2847,10 @@
         <v>119440</v>
       </c>
       <c r="X22" s="61" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y22" s="61" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z22" s="61">
         <v>93.42</v>
@@ -2862,14 +2865,13 @@
         <v>3943.98</v>
       </c>
       <c r="AE22" s="68" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:31" s="46" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:31" s="46" customFormat="1" ht="17" customHeight="1">
       <c r="B23" s="46" t="s">
-        <v>74</v>
-      </c>
-      <c r="J23" s="47"/>
+        <v>70</v>
+      </c>
       <c r="K23" s="48"/>
       <c r="P23" s="47"/>
       <c r="Q23" s="47"/>
@@ -2878,18 +2880,18 @@
       <c r="AD23" s="4"/>
       <c r="AE23" s="69"/>
     </row>
-    <row r="24" spans="1:31" s="4" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:31" s="4" customFormat="1" ht="17" customHeight="1">
       <c r="A24" s="4">
         <v>19</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E24" s="4">
         <v>3</v>
@@ -2907,8 +2909,9 @@
         <f>N24*O24</f>
         <v>1</v>
       </c>
-      <c r="J24" s="26" t="s">
-        <v>77</v>
+      <c r="J24" s="4">
+        <f>G24/F24</f>
+        <v>3.75</v>
       </c>
       <c r="K24" s="17">
         <v>150000</v>
@@ -2926,10 +2929,10 @@
         <v>1</v>
       </c>
       <c r="P24" s="26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="Q24" s="26" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="R24" s="87">
         <v>0.11948499999999999</v>
@@ -2950,33 +2953,33 @@
         <v>97</v>
       </c>
       <c r="X24" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="Y24" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AC24" s="4">
         <v>613.46</v>
       </c>
       <c r="AD24" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE24" s="70" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
-    <row r="25" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:31" s="4" customFormat="1">
       <c r="A25" s="4">
         <v>20</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E25" s="4">
         <v>3</v>
@@ -2991,11 +2994,12 @@
         <v>0.3</v>
       </c>
       <c r="I25" s="4">
-        <f t="shared" ref="I25:I29" si="3">N25*O25</f>
+        <f t="shared" ref="I25:I29" si="6">N25*O25</f>
         <v>1</v>
       </c>
-      <c r="J25" s="26" t="s">
-        <v>77</v>
+      <c r="J25" s="4">
+        <f t="shared" ref="J25:J29" si="7">G25/F25</f>
+        <v>3.75</v>
       </c>
       <c r="K25" s="17">
         <v>150000</v>
@@ -3013,10 +3017,10 @@
         <v>1</v>
       </c>
       <c r="P25" s="26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="Q25" s="26" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="R25" s="87">
         <v>0.112124</v>
@@ -3037,33 +3041,33 @@
         <v>97</v>
       </c>
       <c r="X25" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="Y25" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AC25" s="4">
         <v>678.42</v>
       </c>
       <c r="AD25" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE25" s="70" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
-    <row r="26" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:31" s="4" customFormat="1">
       <c r="A26" s="4">
         <v>21</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E26" s="4">
         <v>3</v>
@@ -3078,11 +3082,12 @@
         <v>0.3</v>
       </c>
       <c r="I26" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="J26" s="26" t="s">
-        <v>77</v>
+      <c r="J26" s="4">
+        <f t="shared" si="7"/>
+        <v>3.75</v>
       </c>
       <c r="K26" s="17">
         <v>150000</v>
@@ -3100,10 +3105,10 @@
         <v>1</v>
       </c>
       <c r="P26" s="26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="Q26" s="26" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="R26" s="87">
         <v>0.153282</v>
@@ -3124,33 +3129,33 @@
         <v>97</v>
       </c>
       <c r="X26" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="Y26" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AC26" s="4">
         <v>53817.56</v>
       </c>
       <c r="AD26" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE26" s="70" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
-    <row r="27" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:31" s="4" customFormat="1">
       <c r="A27" s="4">
         <v>22</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E27" s="4">
         <v>3</v>
@@ -3165,11 +3170,12 @@
         <v>0.3</v>
       </c>
       <c r="I27" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="J27" s="26" t="s">
-        <v>77</v>
+      <c r="J27" s="4">
+        <f t="shared" si="7"/>
+        <v>3.75</v>
       </c>
       <c r="K27" s="17">
         <v>150000</v>
@@ -3187,10 +3193,10 @@
         <v>1</v>
       </c>
       <c r="P27" s="26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="Q27" s="26" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="R27" s="87">
         <v>0.10860400000000001</v>
@@ -3211,33 +3217,33 @@
         <v>98</v>
       </c>
       <c r="X27" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="Y27" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AC27" s="4">
         <v>5369.95</v>
       </c>
       <c r="AD27" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE27" s="70" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
-    <row r="28" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:31" s="4" customFormat="1">
       <c r="A28" s="4">
         <v>23</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="E28" s="4">
         <v>3</v>
@@ -3252,11 +3258,12 @@
         <v>0.3</v>
       </c>
       <c r="I28" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="J28" s="26" t="s">
-        <v>77</v>
+      <c r="J28" s="4">
+        <f t="shared" si="7"/>
+        <v>3.75</v>
       </c>
       <c r="K28" s="17">
         <v>150000</v>
@@ -3275,7 +3282,7 @@
       </c>
       <c r="P28" s="26"/>
       <c r="Q28" s="26" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="R28" s="87">
         <v>2.8732000000000001E-2</v>
@@ -3296,10 +3303,10 @@
         <v>71</v>
       </c>
       <c r="X28" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y28" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z28" s="4">
         <v>0.01</v>
@@ -3314,21 +3321,21 @@
         <v>4.78</v>
       </c>
       <c r="AE28" s="70" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
-    <row r="29" spans="1:31" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:31" s="4" customFormat="1">
       <c r="A29" s="4">
         <v>24</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C29" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="E29" s="4">
         <v>3</v>
@@ -3343,11 +3350,12 @@
         <v>0.3</v>
       </c>
       <c r="I29" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
-      <c r="J29" s="26" t="s">
-        <v>77</v>
+      <c r="J29" s="4">
+        <f t="shared" si="7"/>
+        <v>3.75</v>
       </c>
       <c r="K29" s="17">
         <v>0</v>
@@ -3366,7 +3374,7 @@
       </c>
       <c r="P29" s="26"/>
       <c r="Q29" s="26" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="R29" s="87">
         <v>2.6860999999999999E-2</v>
@@ -3375,10 +3383,10 @@
         <v>0.14255899999999999</v>
       </c>
       <c r="X29" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Y29" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z29" s="4">
         <v>0</v>
@@ -3393,14 +3401,13 @@
         <v>0.03</v>
       </c>
       <c r="AE29" s="70" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:31" s="43" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:31" s="43" customFormat="1">
       <c r="B30" s="43" t="s">
-        <v>92</v>
-      </c>
-      <c r="J30" s="44"/>
+        <v>87</v>
+      </c>
       <c r="K30" s="45"/>
       <c r="P30" s="44"/>
       <c r="Q30" s="44"/>
@@ -3408,18 +3415,18 @@
       <c r="S30" s="88"/>
       <c r="AE30" s="71"/>
     </row>
-    <row r="31" spans="1:31" s="5" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:31" s="5" customFormat="1" ht="17" customHeight="1">
       <c r="A31" s="5">
         <v>26</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E31" s="5">
         <v>8</v>
@@ -3437,8 +3444,9 @@
         <f>N31*O31</f>
         <v>512</v>
       </c>
-      <c r="J31" s="27" t="s">
-        <v>34</v>
+      <c r="J31" s="5">
+        <f>G31/F31</f>
+        <v>10</v>
       </c>
       <c r="K31" s="18">
         <v>0</v>
@@ -3457,7 +3465,7 @@
       </c>
       <c r="P31" s="27"/>
       <c r="Q31" s="27" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R31" s="89">
         <v>2.8E-5</v>
@@ -3466,10 +3474,10 @@
         <v>1.6899999999999999E-4</v>
       </c>
       <c r="X31" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="Y31" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z31" s="5">
         <v>0</v>
@@ -3484,21 +3492,21 @@
         <v>221.77</v>
       </c>
       <c r="AD31" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE31" s="72" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:31" s="5" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:31" s="5" customFormat="1" ht="17" customHeight="1">
       <c r="B32" s="10" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E32" s="5">
         <v>8</v>
@@ -3516,8 +3524,9 @@
         <f>N32*O32</f>
         <v>512</v>
       </c>
-      <c r="J32" s="27" t="s">
-        <v>34</v>
+      <c r="J32" s="5">
+        <f t="shared" ref="J32:J33" si="8">G32/F32</f>
+        <v>10</v>
       </c>
       <c r="K32" s="18">
         <v>131072</v>
@@ -3536,43 +3545,43 @@
       </c>
       <c r="P32" s="27"/>
       <c r="Q32" s="27" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R32" s="90" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="S32" s="90" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="T32" s="32"/>
       <c r="U32" s="32"/>
       <c r="V32" s="32"/>
       <c r="W32" s="32"/>
       <c r="X32" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="Y32" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="AD32" s="5" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="AE32" s="100" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
-    <row r="33" spans="1:31" s="5" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:31" s="5" customFormat="1" ht="17" customHeight="1">
       <c r="A33" s="5">
         <v>27</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E33" s="5">
         <v>8</v>
@@ -3590,8 +3599,9 @@
         <f>N33*O33</f>
         <v>512</v>
       </c>
-      <c r="J33" s="27" t="s">
-        <v>34</v>
+      <c r="J33" s="5">
+        <f t="shared" si="8"/>
+        <v>10</v>
       </c>
       <c r="K33" s="18">
         <v>131072</v>
@@ -3610,7 +3620,7 @@
       </c>
       <c r="P33" s="27"/>
       <c r="Q33" s="27" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R33" s="90">
         <v>1.0512000000000001E-2</v>
@@ -3631,10 +3641,10 @@
         <v>7846</v>
       </c>
       <c r="X33" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="Y33" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z33" s="5">
         <v>15.43</v>
@@ -3649,17 +3659,16 @@
         <v>349.83</v>
       </c>
       <c r="AD33" s="5" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="AE33" s="100" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
-    <row r="34" spans="1:31" s="35" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:31" s="35" customFormat="1">
       <c r="B34" s="36" t="s">
-        <v>101</v>
-      </c>
-      <c r="J34" s="37"/>
+        <v>96</v>
+      </c>
       <c r="K34" s="38"/>
       <c r="P34" s="37"/>
       <c r="Q34" s="37"/>
@@ -3667,18 +3676,18 @@
       <c r="S34" s="92"/>
       <c r="AE34" s="73"/>
     </row>
-    <row r="35" spans="1:31" s="6" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:31" s="6" customFormat="1" ht="17" customHeight="1">
       <c r="A35" s="6">
         <v>28</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E35" s="6">
         <v>8</v>
@@ -3696,8 +3705,9 @@
         <f>N35*O35</f>
         <v>512</v>
       </c>
-      <c r="J35" s="28" t="s">
-        <v>34</v>
+      <c r="J35" s="6">
+        <f>G35/F35</f>
+        <v>10</v>
       </c>
       <c r="K35" s="19">
         <v>131072</v>
@@ -3716,7 +3726,7 @@
       </c>
       <c r="P35" s="28"/>
       <c r="Q35" s="28" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R35" s="93">
         <v>133.57000600000001</v>
@@ -3737,10 +3747,10 @@
         <v>15559</v>
       </c>
       <c r="X35" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y35" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z35" s="6">
         <v>93.11</v>
@@ -3755,24 +3765,24 @@
         <v>801.33</v>
       </c>
       <c r="AD35" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE35" s="74" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:31" s="6" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:31" s="6" customFormat="1" ht="17" customHeight="1">
       <c r="A36" s="6">
         <v>29</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E36" s="6">
         <v>8</v>
@@ -3787,11 +3797,12 @@
         <v>0.1</v>
       </c>
       <c r="I36" s="6">
-        <f t="shared" ref="I36:I38" si="4">N36*O36</f>
+        <f t="shared" ref="I36:I38" si="9">N36*O36</f>
         <v>512</v>
       </c>
-      <c r="J36" s="28" t="s">
-        <v>34</v>
+      <c r="J36" s="6">
+        <f t="shared" ref="J36:J38" si="10">G36/F36</f>
+        <v>10</v>
       </c>
       <c r="K36" s="19">
         <v>131072</v>
@@ -3810,7 +3821,7 @@
       </c>
       <c r="P36" s="28"/>
       <c r="Q36" s="28" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R36" s="93">
         <v>82.246827999999994</v>
@@ -3831,10 +3842,10 @@
         <v>30987</v>
       </c>
       <c r="X36" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y36" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z36" s="6">
         <v>170.98</v>
@@ -3849,24 +3860,24 @@
         <v>1125.3900000000001</v>
       </c>
       <c r="AD36" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE36" s="74" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:31" s="6" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:31" s="6" customFormat="1" ht="17" customHeight="1">
       <c r="A37" s="6">
         <v>30</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E37" s="6">
         <v>8</v>
@@ -3881,11 +3892,12 @@
         <v>0.1</v>
       </c>
       <c r="I37" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>512</v>
       </c>
-      <c r="J37" s="28" t="s">
-        <v>34</v>
+      <c r="J37" s="6">
+        <f t="shared" si="10"/>
+        <v>10</v>
       </c>
       <c r="K37" s="19">
         <v>131072</v>
@@ -3904,7 +3916,7 @@
       </c>
       <c r="P37" s="28"/>
       <c r="Q37" s="28" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R37" s="93">
         <v>0.18355199999999999</v>
@@ -3925,10 +3937,10 @@
         <v>61843</v>
       </c>
       <c r="X37" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y37" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z37" s="6">
         <v>107.53</v>
@@ -3943,24 +3955,24 @@
         <v>4239.91</v>
       </c>
       <c r="AD37" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE37" s="74" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
-    <row r="38" spans="1:31" s="6" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:31" s="6" customFormat="1" ht="17" customHeight="1">
       <c r="A38" s="6">
         <v>31</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E38" s="6">
         <v>8</v>
@@ -3975,11 +3987,12 @@
         <v>0.1</v>
       </c>
       <c r="I38" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>512</v>
       </c>
-      <c r="J38" s="28" t="s">
-        <v>34</v>
+      <c r="J38" s="6">
+        <f t="shared" si="10"/>
+        <v>10</v>
       </c>
       <c r="K38" s="19">
         <v>131072</v>
@@ -3998,7 +4011,7 @@
       </c>
       <c r="P38" s="28"/>
       <c r="Q38" s="28" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R38" s="93">
         <v>7.4400999999999995E-2</v>
@@ -4019,10 +4032,10 @@
         <v>123555</v>
       </c>
       <c r="X38" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y38" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z38" s="6">
         <v>70.45</v>
@@ -4037,17 +4050,16 @@
         <v>92827.3</v>
       </c>
       <c r="AD38" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE38" s="74" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
-    <row r="39" spans="1:31" s="39" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:31" s="39" customFormat="1">
       <c r="B39" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="J39" s="41"/>
+        <v>106</v>
+      </c>
       <c r="K39" s="42"/>
       <c r="P39" s="41"/>
       <c r="Q39" s="41"/>
@@ -4055,18 +4067,18 @@
       <c r="S39" s="94"/>
       <c r="AE39" s="75"/>
     </row>
-    <row r="40" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
       <c r="A40" s="7">
         <v>32</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E40" s="7">
         <v>8</v>
@@ -4084,8 +4096,9 @@
         <f>N40*O40</f>
         <v>512</v>
       </c>
-      <c r="J40" s="29" t="s">
-        <v>34</v>
+      <c r="J40" s="7">
+        <f>G40/F40</f>
+        <v>10</v>
       </c>
       <c r="K40" s="20">
         <v>16384</v>
@@ -4104,7 +4117,7 @@
       </c>
       <c r="P40" s="29"/>
       <c r="Q40" s="29" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R40" s="95">
         <v>60.881906999999998</v>
@@ -4125,10 +4138,10 @@
         <v>61843</v>
       </c>
       <c r="X40" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y40" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z40" s="7">
         <v>298.57</v>
@@ -4143,24 +4156,24 @@
         <v>13247.65</v>
       </c>
       <c r="AD40" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE40" s="76" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
-    <row r="41" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
       <c r="A41" s="7">
         <v>33</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E41" s="7">
         <v>8</v>
@@ -4175,11 +4188,12 @@
         <v>0.1</v>
       </c>
       <c r="I41" s="7">
-        <f t="shared" ref="I41:I44" si="5">N41*O41</f>
+        <f t="shared" ref="I41:I44" si="11">N41*O41</f>
         <v>512</v>
       </c>
-      <c r="J41" s="29" t="s">
-        <v>34</v>
+      <c r="J41" s="7">
+        <f t="shared" ref="J41:J44" si="12">G41/F41</f>
+        <v>10</v>
       </c>
       <c r="K41" s="20">
         <v>65536</v>
@@ -4198,7 +4212,7 @@
       </c>
       <c r="P41" s="29"/>
       <c r="Q41" s="29" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R41" s="95">
         <v>0.199902</v>
@@ -4219,10 +4233,10 @@
         <v>61843</v>
       </c>
       <c r="X41" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y41" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z41" s="7">
         <v>243.68</v>
@@ -4237,24 +4251,24 @@
         <v>13257.85</v>
       </c>
       <c r="AD41" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE41" s="76" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
-    <row r="42" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
       <c r="A42" s="7">
         <v>34</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E42" s="7">
         <v>8</v>
@@ -4269,11 +4283,12 @@
         <v>0.1</v>
       </c>
       <c r="I42" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>512</v>
       </c>
-      <c r="J42" s="29" t="s">
-        <v>34</v>
+      <c r="J42" s="7">
+        <f t="shared" si="12"/>
+        <v>10</v>
       </c>
       <c r="K42" s="20">
         <v>131072</v>
@@ -4292,7 +4307,7 @@
       </c>
       <c r="P42" s="29"/>
       <c r="Q42" s="29" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R42" s="95">
         <v>0.18355199999999999</v>
@@ -4313,10 +4328,10 @@
         <v>61843</v>
       </c>
       <c r="X42" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y42" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z42" s="7">
         <v>285.98</v>
@@ -4331,24 +4346,24 @@
         <v>13257.83</v>
       </c>
       <c r="AD42" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE42" s="76" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
-    <row r="43" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
       <c r="A43" s="7">
         <v>35</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E43" s="7">
         <v>8</v>
@@ -4363,11 +4378,12 @@
         <v>0.1</v>
       </c>
       <c r="I43" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>512</v>
       </c>
-      <c r="J43" s="29" t="s">
-        <v>34</v>
+      <c r="J43" s="7">
+        <f t="shared" si="12"/>
+        <v>10</v>
       </c>
       <c r="K43" s="20">
         <v>524288</v>
@@ -4386,7 +4402,7 @@
       </c>
       <c r="P43" s="29"/>
       <c r="Q43" s="29" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R43" s="95">
         <v>8.6906999999999998E-2</v>
@@ -4407,10 +4423,10 @@
         <v>61843</v>
       </c>
       <c r="X43" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y43" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z43" s="7">
         <v>358.19</v>
@@ -4425,24 +4441,24 @@
         <v>13218.02</v>
       </c>
       <c r="AD43" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE43" s="76" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
-    <row r="44" spans="1:31" s="7" customFormat="1" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:31" s="7" customFormat="1" ht="17" customHeight="1">
       <c r="A44" s="7">
         <v>36</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E44" s="7">
         <v>8</v>
@@ -4457,11 +4473,12 @@
         <v>0.1</v>
       </c>
       <c r="I44" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>512</v>
       </c>
-      <c r="J44" s="29" t="s">
-        <v>34</v>
+      <c r="J44" s="7">
+        <f t="shared" si="12"/>
+        <v>10</v>
       </c>
       <c r="K44" s="20">
         <v>1048576</v>
@@ -4480,7 +4497,7 @@
       </c>
       <c r="P44" s="29"/>
       <c r="Q44" s="29" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="R44" s="95">
         <v>4.7698999999999998E-2</v>
@@ -4501,10 +4518,10 @@
         <v>61843</v>
       </c>
       <c r="X44" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y44" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z44" s="7">
         <v>274.97000000000003</v>
@@ -4519,10 +4536,10 @@
         <v>13259.02</v>
       </c>
       <c r="AD44" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AE44" s="76" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update paper cases table and add FTCS reference-scheme note
Refresh paper_cases_table.xlsx with a dated backup, and document the classical FTCS truth for the QLBM/CH comparison in ftcs_reference_scheme.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aux/burgers-ch-lbm-June2026/paper_cases_table.xlsx
+++ b/aux/burgers-ch-lbm-June2026/paper_cases_table.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Paper cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CH nu-domain (Re sweep)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -4992,4 +4993,4608 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>q</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>nu</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>cfl</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Re</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Shots</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Bond dim</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Phi modes</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>In-segment k</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Segments</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>L2 (rel vs FTCS)</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>cos</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>FTCS ref-points</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>FTCS grid</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>pts/shock (ref)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>wall s</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>results/ dir</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>512</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K2" t="n">
+        <v>512</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>9.000000000000001e-05</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" t="n">
+        <v>800</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>512</v>
+      </c>
+      <c r="R2" t="n">
+        <v>124.8</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/06c51167</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>512</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K3" t="n">
+        <v>512</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.000103</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>800</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>409.6</v>
+      </c>
+      <c r="R3" t="n">
+        <v>125.6</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/fe7a219e</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>512</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" t="n">
+        <v>512</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.000123</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>800</v>
+      </c>
+      <c r="P4" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>273.1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>126</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/348e98f5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>512</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>8</v>
+      </c>
+      <c r="K5" t="n">
+        <v>512</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.000144</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>800</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>170.7</v>
+      </c>
+      <c r="R5" t="n">
+        <v>126.8</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/fd1a816f</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>512</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K6" t="n">
+        <v>512</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.000169</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>800</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="R6" t="n">
+        <v>126.9</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/30cbb15a</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>512</v>
+      </c>
+      <c r="G7" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" t="n">
+        <v>8</v>
+      </c>
+      <c r="K7" t="n">
+        <v>512</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.000187</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>800</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="R7" t="n">
+        <v>125.7</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/9c1fdede</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>512</v>
+      </c>
+      <c r="G8" t="n">
+        <v>20</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4</v>
+      </c>
+      <c r="J8" t="n">
+        <v>8</v>
+      </c>
+      <c r="K8" t="n">
+        <v>512</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.000199</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>800</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="R8" t="n">
+        <v>126.9</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/228678ea</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>512</v>
+      </c>
+      <c r="G9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" t="n">
+        <v>8</v>
+      </c>
+      <c r="K9" t="n">
+        <v>512</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.000216</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>800</v>
+      </c>
+      <c r="P9" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="R9" t="n">
+        <v>126.6</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/e6304c93</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>512</v>
+      </c>
+      <c r="G10" t="n">
+        <v>40</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>8</v>
+      </c>
+      <c r="K10" t="n">
+        <v>512</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.000274</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>800</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="R10" t="n">
+        <v>127</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/f10c17bc</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>512</v>
+      </c>
+      <c r="G11" t="n">
+        <v>60</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" t="n">
+        <v>512</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.001314</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>800</v>
+      </c>
+      <c r="P11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="R11" t="n">
+        <v>126.9</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/1fe02bfd</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>512</v>
+      </c>
+      <c r="G12" t="n">
+        <v>100</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" t="n">
+        <v>8</v>
+      </c>
+      <c r="K12" t="n">
+        <v>512</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.021698</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="O12" t="n">
+        <v>800</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="R12" t="n">
+        <v>125.9</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/7ce83601</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>8</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>512</v>
+      </c>
+      <c r="G13" t="n">
+        <v>120</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4</v>
+      </c>
+      <c r="J13" t="n">
+        <v>8</v>
+      </c>
+      <c r="K13" t="n">
+        <v>512</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.065762</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.9978</v>
+      </c>
+      <c r="O13" t="n">
+        <v>800</v>
+      </c>
+      <c r="P13" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="R13" t="n">
+        <v>125.4</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/9c3d431d</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>8</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>512</v>
+      </c>
+      <c r="G14" t="n">
+        <v>150</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K14" t="n">
+        <v>512</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.401215</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.9298</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1280</v>
+      </c>
+      <c r="P14" t="n">
+        <v>1280</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="R14" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/0db1b897</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>512</v>
+      </c>
+      <c r="G15" t="n">
+        <v>200</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" t="n">
+        <v>8</v>
+      </c>
+      <c r="K15" t="n">
+        <v>512</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>13.292014</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.1025</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1536</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1536</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="R15" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/1119f098</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>512</v>
+      </c>
+      <c r="G16" t="n">
+        <v>300</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" t="n">
+        <v>8</v>
+      </c>
+      <c r="K16" t="n">
+        <v>512</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="n">
+        <v>13.542119</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.0398</v>
+      </c>
+      <c r="O16" t="n">
+        <v>2048</v>
+      </c>
+      <c r="P16" t="n">
+        <v>2048</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R16" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/460ff75e</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>512</v>
+      </c>
+      <c r="G17" t="n">
+        <v>400</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8</v>
+      </c>
+      <c r="K17" t="n">
+        <v>512</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>7.065775</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2816</v>
+      </c>
+      <c r="P17" t="n">
+        <v>2816</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>7</v>
+      </c>
+      <c r="R17" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/3e031de3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>8</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>512</v>
+      </c>
+      <c r="G18" t="n">
+        <v>600</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4</v>
+      </c>
+      <c r="J18" t="n">
+        <v>8</v>
+      </c>
+      <c r="K18" t="n">
+        <v>512</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>5.682078</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="O18" t="n">
+        <v>4096</v>
+      </c>
+      <c r="P18" t="n">
+        <v>4096</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R18" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/7d1bee00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>512</v>
+      </c>
+      <c r="G19" t="n">
+        <v>750</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" t="n">
+        <v>8</v>
+      </c>
+      <c r="K19" t="n">
+        <v>512</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>5.073044</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.0332</v>
+      </c>
+      <c r="O19" t="n">
+        <v>5120</v>
+      </c>
+      <c r="P19" t="n">
+        <v>5120</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R19" t="n">
+        <v>129.4</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/92c74292</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>512</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J20" t="n">
+        <v>8</v>
+      </c>
+      <c r="K20" t="n">
+        <v>512</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" t="n">
+        <v>4.550086</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.0218</v>
+      </c>
+      <c r="O20" t="n">
+        <v>6912</v>
+      </c>
+      <c r="P20" t="n">
+        <v>6912</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="R20" t="n">
+        <v>130.8</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/5c31ff15</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>512</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>4</v>
+      </c>
+      <c r="J21" t="n">
+        <v>8</v>
+      </c>
+      <c r="K21" t="n">
+        <v>512</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" t="n">
+        <v>4.055808</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.0122</v>
+      </c>
+      <c r="O21" t="n">
+        <v>8192</v>
+      </c>
+      <c r="P21" t="n">
+        <v>8192</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R21" t="n">
+        <v>129</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/4431d434</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>8</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>512</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>4</v>
+      </c>
+      <c r="J22" t="n">
+        <v>8</v>
+      </c>
+      <c r="K22" t="n">
+        <v>512</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>3.486151</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.0121</v>
+      </c>
+      <c r="O22" t="n">
+        <v>10240</v>
+      </c>
+      <c r="P22" t="n">
+        <v>10240</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R22" t="n">
+        <v>127.9</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/9614465d</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>8</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.00015</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>512</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>4</v>
+      </c>
+      <c r="J23" t="n">
+        <v>8</v>
+      </c>
+      <c r="K23" t="n">
+        <v>512</v>
+      </c>
+      <c r="L23" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" t="n">
+        <v>2.87503</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.0121</v>
+      </c>
+      <c r="O23" t="n">
+        <v>13568</v>
+      </c>
+      <c r="P23" t="n">
+        <v>13568</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R23" t="n">
+        <v>130</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/fa665f66</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>512</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>8</v>
+      </c>
+      <c r="J24" t="n">
+        <v>8</v>
+      </c>
+      <c r="K24" t="n">
+        <v>512</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" t="n">
+        <v>9.000000000000001e-05</v>
+      </c>
+      <c r="N24" t="n">
+        <v>1</v>
+      </c>
+      <c r="O24" t="n">
+        <v>800</v>
+      </c>
+      <c r="P24" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>512</v>
+      </c>
+      <c r="R24" t="n">
+        <v>126.1</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/300efc8e</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>512</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>8</v>
+      </c>
+      <c r="J25" t="n">
+        <v>8</v>
+      </c>
+      <c r="K25" t="n">
+        <v>512</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.000103</v>
+      </c>
+      <c r="N25" t="n">
+        <v>1</v>
+      </c>
+      <c r="O25" t="n">
+        <v>800</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>409.6</v>
+      </c>
+      <c r="R25" t="n">
+        <v>126.6</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/28063519</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>512</v>
+      </c>
+      <c r="G26" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>8</v>
+      </c>
+      <c r="J26" t="n">
+        <v>8</v>
+      </c>
+      <c r="K26" t="n">
+        <v>512</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.000123</v>
+      </c>
+      <c r="N26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" t="n">
+        <v>800</v>
+      </c>
+      <c r="P26" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>273.1</v>
+      </c>
+      <c r="R26" t="n">
+        <v>126</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/ab5fb73e</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>8</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>512</v>
+      </c>
+      <c r="G27" t="n">
+        <v>6</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>8</v>
+      </c>
+      <c r="J27" t="n">
+        <v>8</v>
+      </c>
+      <c r="K27" t="n">
+        <v>512</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.000144</v>
+      </c>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" t="n">
+        <v>800</v>
+      </c>
+      <c r="P27" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>170.7</v>
+      </c>
+      <c r="R27" t="n">
+        <v>125.7</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/330635af</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>512</v>
+      </c>
+      <c r="G28" t="n">
+        <v>10</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>8</v>
+      </c>
+      <c r="J28" t="n">
+        <v>8</v>
+      </c>
+      <c r="K28" t="n">
+        <v>512</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.000169</v>
+      </c>
+      <c r="N28" t="n">
+        <v>1</v>
+      </c>
+      <c r="O28" t="n">
+        <v>800</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="R28" t="n">
+        <v>127.1</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/94e8ac7b</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>8</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>512</v>
+      </c>
+      <c r="G29" t="n">
+        <v>15</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>8</v>
+      </c>
+      <c r="J29" t="n">
+        <v>8</v>
+      </c>
+      <c r="K29" t="n">
+        <v>512</v>
+      </c>
+      <c r="L29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.000187</v>
+      </c>
+      <c r="N29" t="n">
+        <v>1</v>
+      </c>
+      <c r="O29" t="n">
+        <v>800</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="R29" t="n">
+        <v>126.2</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/7540deb4</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>8</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>512</v>
+      </c>
+      <c r="G30" t="n">
+        <v>20</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>8</v>
+      </c>
+      <c r="J30" t="n">
+        <v>8</v>
+      </c>
+      <c r="K30" t="n">
+        <v>512</v>
+      </c>
+      <c r="L30" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0.000199</v>
+      </c>
+      <c r="N30" t="n">
+        <v>1</v>
+      </c>
+      <c r="O30" t="n">
+        <v>800</v>
+      </c>
+      <c r="P30" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="R30" t="n">
+        <v>125.5</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/275a1e38</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>8</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>512</v>
+      </c>
+      <c r="G31" t="n">
+        <v>30</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>8</v>
+      </c>
+      <c r="J31" t="n">
+        <v>8</v>
+      </c>
+      <c r="K31" t="n">
+        <v>512</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.000213</v>
+      </c>
+      <c r="N31" t="n">
+        <v>1</v>
+      </c>
+      <c r="O31" t="n">
+        <v>800</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="R31" t="n">
+        <v>127</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/31f791e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>512</v>
+      </c>
+      <c r="G32" t="n">
+        <v>40</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>8</v>
+      </c>
+      <c r="J32" t="n">
+        <v>8</v>
+      </c>
+      <c r="K32" t="n">
+        <v>512</v>
+      </c>
+      <c r="L32" t="n">
+        <v>1</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.000227</v>
+      </c>
+      <c r="N32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" t="n">
+        <v>800</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="R32" t="n">
+        <v>127</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/9f687915</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>8</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>512</v>
+      </c>
+      <c r="G33" t="n">
+        <v>60</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>8</v>
+      </c>
+      <c r="J33" t="n">
+        <v>8</v>
+      </c>
+      <c r="K33" t="n">
+        <v>512</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.000289</v>
+      </c>
+      <c r="N33" t="n">
+        <v>1</v>
+      </c>
+      <c r="O33" t="n">
+        <v>800</v>
+      </c>
+      <c r="P33" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="R33" t="n">
+        <v>126.6</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/a2831fc2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>8</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>512</v>
+      </c>
+      <c r="G34" t="n">
+        <v>100</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>8</v>
+      </c>
+      <c r="J34" t="n">
+        <v>8</v>
+      </c>
+      <c r="K34" t="n">
+        <v>512</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.0006310000000000001</v>
+      </c>
+      <c r="N34" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" t="n">
+        <v>800</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="R34" t="n">
+        <v>126.9</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/4284386d</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>8</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>512</v>
+      </c>
+      <c r="G35" t="n">
+        <v>120</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="n">
+        <v>8</v>
+      </c>
+      <c r="J35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K35" t="n">
+        <v>512</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.000899</v>
+      </c>
+      <c r="N35" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" t="n">
+        <v>800</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="R35" t="n">
+        <v>126.1</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/4aacc4bd</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>8</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>512</v>
+      </c>
+      <c r="G36" t="n">
+        <v>150</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>8</v>
+      </c>
+      <c r="J36" t="n">
+        <v>8</v>
+      </c>
+      <c r="K36" t="n">
+        <v>512</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.001474</v>
+      </c>
+      <c r="N36" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1280</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1280</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="R36" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/859a069e</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>8</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>512</v>
+      </c>
+      <c r="G37" t="n">
+        <v>200</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>8</v>
+      </c>
+      <c r="J37" t="n">
+        <v>8</v>
+      </c>
+      <c r="K37" t="n">
+        <v>512</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.231955</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0.9728</v>
+      </c>
+      <c r="O37" t="n">
+        <v>1536</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1536</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="R37" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/7ea4ec41</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>8</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>512</v>
+      </c>
+      <c r="G38" t="n">
+        <v>300</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="n">
+        <v>8</v>
+      </c>
+      <c r="J38" t="n">
+        <v>8</v>
+      </c>
+      <c r="K38" t="n">
+        <v>512</v>
+      </c>
+      <c r="L38" t="n">
+        <v>1</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.6360789999999999</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0.7716</v>
+      </c>
+      <c r="O38" t="n">
+        <v>2048</v>
+      </c>
+      <c r="P38" t="n">
+        <v>2048</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R38" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>marginal</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/ef257f64</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>512</v>
+      </c>
+      <c r="G39" t="n">
+        <v>400</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>8</v>
+      </c>
+      <c r="J39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K39" t="n">
+        <v>512</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0.775056</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0.632</v>
+      </c>
+      <c r="O39" t="n">
+        <v>2816</v>
+      </c>
+      <c r="P39" t="n">
+        <v>2816</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>7</v>
+      </c>
+      <c r="R39" t="n">
+        <v>47</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>marginal</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/9e91f02d</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>8</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>512</v>
+      </c>
+      <c r="G40" t="n">
+        <v>600</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="n">
+        <v>8</v>
+      </c>
+      <c r="J40" t="n">
+        <v>8</v>
+      </c>
+      <c r="K40" t="n">
+        <v>512</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" t="n">
+        <v>3.612818</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="O40" t="n">
+        <v>4096</v>
+      </c>
+      <c r="P40" t="n">
+        <v>4096</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R40" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/60ece56b</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>8</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F41" t="n">
+        <v>512</v>
+      </c>
+      <c r="G41" t="n">
+        <v>750</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>8</v>
+      </c>
+      <c r="J41" t="n">
+        <v>8</v>
+      </c>
+      <c r="K41" t="n">
+        <v>512</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" t="n">
+        <v>3.677275</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0.0486</v>
+      </c>
+      <c r="O41" t="n">
+        <v>5120</v>
+      </c>
+      <c r="P41" t="n">
+        <v>5120</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R41" t="n">
+        <v>129.6</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/5b100faf</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>8</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>512</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>8</v>
+      </c>
+      <c r="J42" t="n">
+        <v>8</v>
+      </c>
+      <c r="K42" t="n">
+        <v>512</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" t="n">
+        <v>3.545545</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.0349</v>
+      </c>
+      <c r="O42" t="n">
+        <v>6912</v>
+      </c>
+      <c r="P42" t="n">
+        <v>6912</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="R42" t="n">
+        <v>126.3</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/52461db0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>8</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>512</v>
+      </c>
+      <c r="G43" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>8</v>
+      </c>
+      <c r="J43" t="n">
+        <v>8</v>
+      </c>
+      <c r="K43" t="n">
+        <v>512</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1</v>
+      </c>
+      <c r="M43" t="n">
+        <v>3.008312</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0.0322</v>
+      </c>
+      <c r="O43" t="n">
+        <v>8192</v>
+      </c>
+      <c r="P43" t="n">
+        <v>8192</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R43" t="n">
+        <v>129.9</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/8c78a249</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>512</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>8</v>
+      </c>
+      <c r="J44" t="n">
+        <v>8</v>
+      </c>
+      <c r="K44" t="n">
+        <v>512</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" t="n">
+        <v>3.325335</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0.0248</v>
+      </c>
+      <c r="O44" t="n">
+        <v>10240</v>
+      </c>
+      <c r="P44" t="n">
+        <v>10240</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R44" t="n">
+        <v>128.5</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/d07b3bea</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>8</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0.00015</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>512</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>8</v>
+      </c>
+      <c r="J45" t="n">
+        <v>8</v>
+      </c>
+      <c r="K45" t="n">
+        <v>512</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1</v>
+      </c>
+      <c r="M45" t="n">
+        <v>2.605501</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="O45" t="n">
+        <v>13568</v>
+      </c>
+      <c r="P45" t="n">
+        <v>13568</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R45" t="n">
+        <v>128.3</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/95945d0a</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>8</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F46" t="n">
+        <v>512</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>16</v>
+      </c>
+      <c r="J46" t="n">
+        <v>8</v>
+      </c>
+      <c r="K46" t="n">
+        <v>512</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1</v>
+      </c>
+      <c r="M46" t="n">
+        <v>9.000000000000001e-05</v>
+      </c>
+      <c r="N46" t="n">
+        <v>1</v>
+      </c>
+      <c r="O46" t="n">
+        <v>800</v>
+      </c>
+      <c r="P46" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>512</v>
+      </c>
+      <c r="R46" t="n">
+        <v>125.6</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/72818197</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>8</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>512</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>16</v>
+      </c>
+      <c r="J47" t="n">
+        <v>8</v>
+      </c>
+      <c r="K47" t="n">
+        <v>512</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0.000103</v>
+      </c>
+      <c r="N47" t="n">
+        <v>1</v>
+      </c>
+      <c r="O47" t="n">
+        <v>800</v>
+      </c>
+      <c r="P47" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>409.6</v>
+      </c>
+      <c r="R47" t="n">
+        <v>127.3</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/63cf775c</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>8</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>512</v>
+      </c>
+      <c r="G48" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>16</v>
+      </c>
+      <c r="J48" t="n">
+        <v>8</v>
+      </c>
+      <c r="K48" t="n">
+        <v>512</v>
+      </c>
+      <c r="L48" t="n">
+        <v>1</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0.000123</v>
+      </c>
+      <c r="N48" t="n">
+        <v>1</v>
+      </c>
+      <c r="O48" t="n">
+        <v>800</v>
+      </c>
+      <c r="P48" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>273.1</v>
+      </c>
+      <c r="R48" t="n">
+        <v>126.9</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/3550a3b2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>8</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>512</v>
+      </c>
+      <c r="G49" t="n">
+        <v>6</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="n">
+        <v>16</v>
+      </c>
+      <c r="J49" t="n">
+        <v>8</v>
+      </c>
+      <c r="K49" t="n">
+        <v>512</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0.000144</v>
+      </c>
+      <c r="N49" t="n">
+        <v>1</v>
+      </c>
+      <c r="O49" t="n">
+        <v>800</v>
+      </c>
+      <c r="P49" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>170.7</v>
+      </c>
+      <c r="R49" t="n">
+        <v>126.3</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/3b65b1ff</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>8</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F50" t="n">
+        <v>512</v>
+      </c>
+      <c r="G50" t="n">
+        <v>10</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="n">
+        <v>16</v>
+      </c>
+      <c r="J50" t="n">
+        <v>8</v>
+      </c>
+      <c r="K50" t="n">
+        <v>512</v>
+      </c>
+      <c r="L50" t="n">
+        <v>1</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0.000169</v>
+      </c>
+      <c r="N50" t="n">
+        <v>1</v>
+      </c>
+      <c r="O50" t="n">
+        <v>800</v>
+      </c>
+      <c r="P50" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="R50" t="n">
+        <v>126.8</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/9951b427</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>8</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>512</v>
+      </c>
+      <c r="G51" t="n">
+        <v>15</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="n">
+        <v>16</v>
+      </c>
+      <c r="J51" t="n">
+        <v>8</v>
+      </c>
+      <c r="K51" t="n">
+        <v>512</v>
+      </c>
+      <c r="L51" t="n">
+        <v>1</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0.000187</v>
+      </c>
+      <c r="N51" t="n">
+        <v>1</v>
+      </c>
+      <c r="O51" t="n">
+        <v>800</v>
+      </c>
+      <c r="P51" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="R51" t="n">
+        <v>126</v>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/be363365</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>8</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F52" t="n">
+        <v>512</v>
+      </c>
+      <c r="G52" t="n">
+        <v>20</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="n">
+        <v>16</v>
+      </c>
+      <c r="J52" t="n">
+        <v>8</v>
+      </c>
+      <c r="K52" t="n">
+        <v>512</v>
+      </c>
+      <c r="L52" t="n">
+        <v>1</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0.000199</v>
+      </c>
+      <c r="N52" t="n">
+        <v>1</v>
+      </c>
+      <c r="O52" t="n">
+        <v>800</v>
+      </c>
+      <c r="P52" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="R52" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/71059e23</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>8</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>512</v>
+      </c>
+      <c r="G53" t="n">
+        <v>30</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="n">
+        <v>16</v>
+      </c>
+      <c r="J53" t="n">
+        <v>8</v>
+      </c>
+      <c r="K53" t="n">
+        <v>512</v>
+      </c>
+      <c r="L53" t="n">
+        <v>1</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0.000213</v>
+      </c>
+      <c r="N53" t="n">
+        <v>1</v>
+      </c>
+      <c r="O53" t="n">
+        <v>800</v>
+      </c>
+      <c r="P53" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="R53" t="n">
+        <v>126.8</v>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/0195ba52</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>8</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>512</v>
+      </c>
+      <c r="G54" t="n">
+        <v>40</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="n">
+        <v>16</v>
+      </c>
+      <c r="J54" t="n">
+        <v>8</v>
+      </c>
+      <c r="K54" t="n">
+        <v>512</v>
+      </c>
+      <c r="L54" t="n">
+        <v>1</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.000227</v>
+      </c>
+      <c r="N54" t="n">
+        <v>1</v>
+      </c>
+      <c r="O54" t="n">
+        <v>800</v>
+      </c>
+      <c r="P54" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="R54" t="n">
+        <v>124.4</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/d2688e31</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>8</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>512</v>
+      </c>
+      <c r="G55" t="n">
+        <v>60</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="n">
+        <v>16</v>
+      </c>
+      <c r="J55" t="n">
+        <v>8</v>
+      </c>
+      <c r="K55" t="n">
+        <v>512</v>
+      </c>
+      <c r="L55" t="n">
+        <v>1</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0.000289</v>
+      </c>
+      <c r="N55" t="n">
+        <v>1</v>
+      </c>
+      <c r="O55" t="n">
+        <v>800</v>
+      </c>
+      <c r="P55" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="R55" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/7cc4209a</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>8</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>512</v>
+      </c>
+      <c r="G56" t="n">
+        <v>100</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="n">
+        <v>16</v>
+      </c>
+      <c r="J56" t="n">
+        <v>8</v>
+      </c>
+      <c r="K56" t="n">
+        <v>512</v>
+      </c>
+      <c r="L56" t="n">
+        <v>1</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0.0006310000000000001</v>
+      </c>
+      <c r="N56" t="n">
+        <v>1</v>
+      </c>
+      <c r="O56" t="n">
+        <v>800</v>
+      </c>
+      <c r="P56" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="R56" t="n">
+        <v>127.1</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/d784896b</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>8</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>512</v>
+      </c>
+      <c r="G57" t="n">
+        <v>120</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="n">
+        <v>16</v>
+      </c>
+      <c r="J57" t="n">
+        <v>8</v>
+      </c>
+      <c r="K57" t="n">
+        <v>512</v>
+      </c>
+      <c r="L57" t="n">
+        <v>1</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0.000899</v>
+      </c>
+      <c r="N57" t="n">
+        <v>1</v>
+      </c>
+      <c r="O57" t="n">
+        <v>800</v>
+      </c>
+      <c r="P57" t="n">
+        <v>1024</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="R57" t="n">
+        <v>126.7</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_ce436320/41597ce5</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>8</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F58" t="n">
+        <v>512</v>
+      </c>
+      <c r="G58" t="n">
+        <v>150</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>16</v>
+      </c>
+      <c r="J58" t="n">
+        <v>8</v>
+      </c>
+      <c r="K58" t="n">
+        <v>512</v>
+      </c>
+      <c r="L58" t="n">
+        <v>1</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0.00147</v>
+      </c>
+      <c r="N58" t="n">
+        <v>1</v>
+      </c>
+      <c r="O58" t="n">
+        <v>1280</v>
+      </c>
+      <c r="P58" t="n">
+        <v>1280</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="R58" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/79da63cf</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>8</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F59" t="n">
+        <v>512</v>
+      </c>
+      <c r="G59" t="n">
+        <v>200</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="n">
+        <v>16</v>
+      </c>
+      <c r="J59" t="n">
+        <v>8</v>
+      </c>
+      <c r="K59" t="n">
+        <v>512</v>
+      </c>
+      <c r="L59" t="n">
+        <v>1</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0.231629</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0.9729</v>
+      </c>
+      <c r="O59" t="n">
+        <v>1536</v>
+      </c>
+      <c r="P59" t="n">
+        <v>1536</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="R59" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/8b142d3e</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>8</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F60" t="n">
+        <v>512</v>
+      </c>
+      <c r="G60" t="n">
+        <v>300</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="n">
+        <v>16</v>
+      </c>
+      <c r="J60" t="n">
+        <v>8</v>
+      </c>
+      <c r="K60" t="n">
+        <v>512</v>
+      </c>
+      <c r="L60" t="n">
+        <v>1</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0.634296</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0.7731</v>
+      </c>
+      <c r="O60" t="n">
+        <v>2048</v>
+      </c>
+      <c r="P60" t="n">
+        <v>2048</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R60" t="n">
+        <v>46</v>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>marginal</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/bf317613</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>8</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0.00075</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F61" t="n">
+        <v>512</v>
+      </c>
+      <c r="G61" t="n">
+        <v>400</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" t="n">
+        <v>16</v>
+      </c>
+      <c r="J61" t="n">
+        <v>8</v>
+      </c>
+      <c r="K61" t="n">
+        <v>512</v>
+      </c>
+      <c r="L61" t="n">
+        <v>1</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0.7766690000000001</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0.6301</v>
+      </c>
+      <c r="O61" t="n">
+        <v>2816</v>
+      </c>
+      <c r="P61" t="n">
+        <v>2816</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>7</v>
+      </c>
+      <c r="R61" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>marginal</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/305cbd15</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>8</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F62" t="n">
+        <v>512</v>
+      </c>
+      <c r="G62" t="n">
+        <v>600</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="n">
+        <v>16</v>
+      </c>
+      <c r="J62" t="n">
+        <v>8</v>
+      </c>
+      <c r="K62" t="n">
+        <v>512</v>
+      </c>
+      <c r="L62" t="n">
+        <v>1</v>
+      </c>
+      <c r="M62" t="n">
+        <v>3.619276</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0.0663</v>
+      </c>
+      <c r="O62" t="n">
+        <v>4096</v>
+      </c>
+      <c r="P62" t="n">
+        <v>4096</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R62" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_83f4f49e/ce4bd185</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>8</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F63" t="n">
+        <v>512</v>
+      </c>
+      <c r="G63" t="n">
+        <v>750</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>16</v>
+      </c>
+      <c r="J63" t="n">
+        <v>8</v>
+      </c>
+      <c r="K63" t="n">
+        <v>512</v>
+      </c>
+      <c r="L63" t="n">
+        <v>1</v>
+      </c>
+      <c r="M63" t="n">
+        <v>3.693238</v>
+      </c>
+      <c r="N63" t="n">
+        <v>0.0486</v>
+      </c>
+      <c r="O63" t="n">
+        <v>5120</v>
+      </c>
+      <c r="P63" t="n">
+        <v>5120</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R63" t="n">
+        <v>127.2</v>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/6f487a2c</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>8</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F64" t="n">
+        <v>512</v>
+      </c>
+      <c r="G64" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="n">
+        <v>16</v>
+      </c>
+      <c r="J64" t="n">
+        <v>8</v>
+      </c>
+      <c r="K64" t="n">
+        <v>512</v>
+      </c>
+      <c r="L64" t="n">
+        <v>1</v>
+      </c>
+      <c r="M64" t="n">
+        <v>4.090417</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="O64" t="n">
+        <v>6912</v>
+      </c>
+      <c r="P64" t="n">
+        <v>6912</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="R64" t="n">
+        <v>126.7</v>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/17f17789</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>8</v>
+      </c>
+      <c r="C65" t="n">
+        <v>0.00025</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F65" t="n">
+        <v>512</v>
+      </c>
+      <c r="G65" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="n">
+        <v>16</v>
+      </c>
+      <c r="J65" t="n">
+        <v>8</v>
+      </c>
+      <c r="K65" t="n">
+        <v>512</v>
+      </c>
+      <c r="L65" t="n">
+        <v>1</v>
+      </c>
+      <c r="M65" t="n">
+        <v>3.460696</v>
+      </c>
+      <c r="N65" t="n">
+        <v>0.0289</v>
+      </c>
+      <c r="O65" t="n">
+        <v>8192</v>
+      </c>
+      <c r="P65" t="n">
+        <v>8192</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R65" t="n">
+        <v>129.6</v>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/dd4ce212</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>8</v>
+      </c>
+      <c r="C66" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F66" t="n">
+        <v>512</v>
+      </c>
+      <c r="G66" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>16</v>
+      </c>
+      <c r="J66" t="n">
+        <v>8</v>
+      </c>
+      <c r="K66" t="n">
+        <v>512</v>
+      </c>
+      <c r="L66" t="n">
+        <v>1</v>
+      </c>
+      <c r="M66" t="n">
+        <v>3.322622</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0.0251</v>
+      </c>
+      <c r="O66" t="n">
+        <v>10240</v>
+      </c>
+      <c r="P66" t="n">
+        <v>10240</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R66" t="n">
+        <v>127.9</v>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/c3cab13a</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>8</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0.00015</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F67" t="n">
+        <v>512</v>
+      </c>
+      <c r="G67" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="n">
+        <v>16</v>
+      </c>
+      <c r="J67" t="n">
+        <v>8</v>
+      </c>
+      <c r="K67" t="n">
+        <v>512</v>
+      </c>
+      <c r="L67" t="n">
+        <v>1</v>
+      </c>
+      <c r="M67" t="n">
+        <v>2.609227</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0.0209</v>
+      </c>
+      <c r="O67" t="n">
+        <v>13568</v>
+      </c>
+      <c r="P67" t="n">
+        <v>13568</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="R67" t="n">
+        <v>128</v>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>diverged</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/22778859</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
rerun of fig 1 with new code
</commit_message>
<xml_diff>
--- a/aux/burgers-ch-lbm-June2026/paper_cases_table.xlsx
+++ b/aux/burgers-ch-lbm-June2026/paper_cases_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\223107543\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{952967B6-94D9-4459-B498-C412A56F66A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7AAF73E-5E88-4660-B780-51E503C18BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="235">
   <si>
     <t>#</t>
   </si>
@@ -471,6 +471,48 @@
     <t>burgers-ch-lbm/ch_q8_c1B/2026-09-02/_2ce06310/8e58998d</t>
   </si>
   <si>
+    <t>IBM Aer sim (AWS Batch)</t>
+  </si>
+  <si>
+    <t>AWS Batch</t>
+  </si>
+  <si>
+    <t>Collapse rerun of case 1 (CH q4). Collapse ON: 7 q / depth 808 / 247 CX vs June 10 q / 3046 / 1006 CX. L2 = final-frame canonical relL2 (||a-b||/||b||, make_plots_vs_ftcs.py), NOT the June Fig.1 plotting-pipeline metric — do not read a CH regression vs rows 3-8.</t>
+  </si>
+  <si>
+    <t>burgers-ch-lbm/ch_fig1_ab_mutual_q4/2026-09-03/_0daaf069/b7509f5c</t>
+  </si>
+  <si>
+    <t>Collapse rerun of case 2 (CH q6): 10 q / depth 4438 / 1606 CX vs June 14 q / 16602 / 6628 CX. L2 = final-frame canonical relL2 (||a-b||/||b||, make_plots_vs_ftcs.py), NOT the June Fig.1 plotting-pipeline metric — do not read a CH regression vs rows 3-8.</t>
+  </si>
+  <si>
+    <t>burgers-ch-lbm/ch_fig1_ab_mutual_q6/2026-09-03/_d61160a7/90fe44cd</t>
+  </si>
+  <si>
+    <t>Collapse rerun of case 4 (QLBM q4). QLBM path untouched by collapse: circuit identical to June (9 q / 119440 CX) and relL2 0.6043 bit-reproduces June. tau=0.98&lt;=1 at N=16 =&gt; QALB divergent regime (expected degradation, not a failure).</t>
+  </si>
+  <si>
+    <t>burgers-ch-lbm/ch_fig1_ab_mutual_q4/2026-09-03/_0daaf069/42a3615a</t>
+  </si>
+  <si>
+    <t>Collapse rerun of case 5 (QLBM q6). QLBM untouched by collapse; circuit identical to June, relL2 0.0985 recovers (tau=2.42, out of divergent regime).</t>
+  </si>
+  <si>
+    <t>burgers-ch-lbm/ch_fig1_ab_mutual_q6/2026-09-03/_d61160a7/2c2561e4</t>
+  </si>
+  <si>
+    <t>Collapse rerun of case 3 (CH q8). Collapse ON: 13 q / depth 21944 / 9416 CX vs June 17 q / 84156 / 40272 CX (~4.3x fewer 2q gates). DIVERGED at this op point: relL2 1.615, u_final overshoots to +1.12/-0.79 vs physical +/-0.25 -- bit-reproduces June's diverged CH q8 (row 5), a known-bad point, NOT a new failure. L2 = final-frame canonical relL2 (||a-b||/||b||, make_plots_vs_ftcs.py). (matches row 5 exactly here.)</t>
+  </si>
+  <si>
+    <t>burgers-ch-lbm/ch_fig1_ab_mutual_q8/2026-09-03/_3da12f29/7fd5a918</t>
+  </si>
+  <si>
+    <t>Collapse rerun of case 6 (QLBM q8). QLBM untouched by collapse: circuit identical to June (9 q / 119440 CX) and relL2 0.3275 bit-reproduces June (tau=8.18, healthy). Wall 3401 s dominated by 10240 dense-collision circuits.</t>
+  </si>
+  <si>
+    <t>burgers-ch-lbm/ch_fig1_ab_mutual_q8/2026-09-03/_3da12f29/4ab5be3a</t>
+  </si>
+  <si>
     <t>L2 (rel vs FTCS)</t>
   </si>
   <si>
@@ -694,6 +736,9 @@
   </si>
   <si>
     <t>results/burgers-ch-lbm/ch_q8_nu_domain_single/2026-09-02/_c2442f4c/22778859</t>
+  </si>
+  <si>
+    <t>Fig. 1 rerun (collapse code): CH &amp; QLBM/QALB</t>
   </si>
 </sst>
 </file>
@@ -835,7 +880,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1002,6 +1047,13 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1336,7 +1388,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE55"/>
+  <dimension ref="A1:AE62"/>
   <sheetFormatPr defaultColWidth="10.84765625" defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="4.1484375" style="8" customWidth="1"/>
@@ -1365,8 +1417,8 @@
     <col min="29" max="29" width="11.1484375" style="8" customWidth="1"/>
     <col min="30" max="30" width="19.34765625" style="8" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="89.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.84765625" style="8" customWidth="1"/>
-    <col min="34" max="16384" width="10.84765625" style="8"/>
+    <col min="32" max="34" width="10.84765625" style="8" customWidth="1"/>
+    <col min="35" max="16384" width="10.84765625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31" s="9" customFormat="1" ht="17.05" customHeight="1" x14ac:dyDescent="0.6">
@@ -4994,9 +5046,7 @@
         <v>256</v>
       </c>
       <c r="P47" s="28"/>
-      <c r="Q47" s="28" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q47" s="28"/>
       <c r="R47" s="93">
         <v>133.57000600000001</v>
       </c>
@@ -5086,9 +5136,7 @@
         <v>128</v>
       </c>
       <c r="P48" s="28"/>
-      <c r="Q48" s="28" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q48" s="28"/>
       <c r="R48" s="93">
         <v>82.246827999999994</v>
       </c>
@@ -5181,9 +5229,7 @@
         <v>64</v>
       </c>
       <c r="P49" s="28"/>
-      <c r="Q49" s="28" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q49" s="28"/>
       <c r="R49" s="93">
         <v>0.18355199999999999</v>
       </c>
@@ -5276,9 +5322,7 @@
         <v>32</v>
       </c>
       <c r="P50" s="28"/>
-      <c r="Q50" s="28" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q50" s="28"/>
       <c r="R50" s="93">
         <v>7.4400999999999995E-2</v>
       </c>
@@ -5371,9 +5415,7 @@
         <v>16</v>
       </c>
       <c r="P51" s="28"/>
-      <c r="Q51" s="28" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q51" s="28"/>
       <c r="R51" s="93">
         <v>4.138E-2</v>
       </c>
@@ -5466,9 +5508,7 @@
         <v>8</v>
       </c>
       <c r="P52" s="28"/>
-      <c r="Q52" s="28" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q52" s="28"/>
       <c r="R52" s="93">
         <v>2.6450999999999999E-2</v>
       </c>
@@ -5561,9 +5601,7 @@
         <v>4</v>
       </c>
       <c r="P53" s="28"/>
-      <c r="Q53" s="28" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q53" s="28"/>
       <c r="R53" s="93">
         <v>1.7378999999999999E-2</v>
       </c>
@@ -5656,9 +5694,7 @@
         <v>2</v>
       </c>
       <c r="P54" s="28"/>
-      <c r="Q54" s="28" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q54" s="28"/>
       <c r="R54" s="93">
         <v>1.5134999999999999E-2</v>
       </c>
@@ -5751,9 +5787,7 @@
         <v>1</v>
       </c>
       <c r="P55" s="28"/>
-      <c r="Q55" s="28" t="s">
-        <v>92</v>
-      </c>
+      <c r="Q55" s="28"/>
       <c r="R55" s="93">
         <v>1.0512000000000001E-2</v>
       </c>
@@ -5795,6 +5829,573 @@
       </c>
       <c r="AE55" s="74" t="s">
         <v>144</v>
+      </c>
+    </row>
+    <row r="56" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.6">
+      <c r="B56" s="104" t="s">
+        <v>234</v>
+      </c>
+      <c r="K56" s="14"/>
+      <c r="P56" s="23"/>
+      <c r="Q56" s="23"/>
+      <c r="R56" s="81"/>
+      <c r="S56" s="102"/>
+      <c r="T56" s="103"/>
+      <c r="U56" s="103"/>
+      <c r="V56" s="103"/>
+      <c r="W56" s="103"/>
+      <c r="Y56" s="64"/>
+    </row>
+    <row r="57" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.6">
+      <c r="A57" s="1">
+        <v>46</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E57" s="1">
+        <v>4</v>
+      </c>
+      <c r="F57" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="G57" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="H57" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="I57" s="1">
+        <f t="shared" ref="I57:I61" si="10">N57*O57</f>
+        <v>30</v>
+      </c>
+      <c r="J57" s="1">
+        <f t="shared" ref="J57:J61" si="11">G57/F57</f>
+        <v>10</v>
+      </c>
+      <c r="K57" s="1">
+        <v>150000</v>
+      </c>
+      <c r="L57" s="1">
+        <v>8</v>
+      </c>
+      <c r="M57" s="1">
+        <v>8</v>
+      </c>
+      <c r="N57" s="1">
+        <v>5</v>
+      </c>
+      <c r="O57" s="1">
+        <v>6</v>
+      </c>
+      <c r="P57" s="23"/>
+      <c r="R57" s="1">
+        <v>2.2023000000000001E-2</v>
+      </c>
+      <c r="S57" s="1">
+        <v>0.13011300000000001</v>
+      </c>
+      <c r="T57" s="1">
+        <v>7</v>
+      </c>
+      <c r="U57" s="1">
+        <v>808</v>
+      </c>
+      <c r="V57" s="1">
+        <v>1103</v>
+      </c>
+      <c r="W57" s="1">
+        <v>247</v>
+      </c>
+      <c r="X57" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y57" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z57" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="AA57" s="1">
+        <v>0.31</v>
+      </c>
+      <c r="AB57" s="1">
+        <v>0.63</v>
+      </c>
+      <c r="AC57" s="1">
+        <v>4.53</v>
+      </c>
+      <c r="AD57" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="AE57" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="58" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.6">
+      <c r="A58" s="1">
+        <v>47</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E58" s="1">
+        <v>6</v>
+      </c>
+      <c r="F58" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="G58" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="H58" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="I58" s="1">
+        <f>N58*O58</f>
+        <v>100</v>
+      </c>
+      <c r="J58" s="1">
+        <f>G58/F58</f>
+        <v>10</v>
+      </c>
+      <c r="K58" s="1">
+        <v>150000</v>
+      </c>
+      <c r="L58" s="1">
+        <v>8</v>
+      </c>
+      <c r="M58" s="1">
+        <v>8</v>
+      </c>
+      <c r="N58" s="1">
+        <v>5</v>
+      </c>
+      <c r="O58" s="1">
+        <v>20</v>
+      </c>
+      <c r="P58" s="23"/>
+      <c r="R58" s="1">
+        <v>5.1749000000000003E-2</v>
+      </c>
+      <c r="S58" s="1">
+        <v>0.294238</v>
+      </c>
+      <c r="T58" s="1">
+        <v>10</v>
+      </c>
+      <c r="U58" s="1">
+        <v>4438</v>
+      </c>
+      <c r="V58" s="1">
+        <v>6309</v>
+      </c>
+      <c r="W58" s="1">
+        <v>1606</v>
+      </c>
+      <c r="X58" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y58" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z58" s="1">
+        <v>0.46</v>
+      </c>
+      <c r="AA58" s="1">
+        <v>1.26</v>
+      </c>
+      <c r="AB58" s="1">
+        <v>2.81</v>
+      </c>
+      <c r="AC58" s="1">
+        <v>11.69</v>
+      </c>
+      <c r="AD58" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AE58" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="59" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.6">
+      <c r="A59" s="1">
+        <v>50</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E59" s="1">
+        <v>8</v>
+      </c>
+      <c r="F59" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="G59" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="H59" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="I59" s="1">
+        <f>N59*O59</f>
+        <v>400</v>
+      </c>
+      <c r="J59" s="1">
+        <f>G59/F59</f>
+        <v>10</v>
+      </c>
+      <c r="K59" s="1">
+        <v>150000</v>
+      </c>
+      <c r="L59" s="1">
+        <v>16</v>
+      </c>
+      <c r="M59" s="1">
+        <v>8</v>
+      </c>
+      <c r="N59" s="1">
+        <v>5</v>
+      </c>
+      <c r="O59" s="1">
+        <v>80</v>
+      </c>
+      <c r="P59" s="23"/>
+      <c r="R59" s="1">
+        <v>0.28409899999999999</v>
+      </c>
+      <c r="S59" s="1">
+        <v>1.6153379999999999</v>
+      </c>
+      <c r="T59" s="1">
+        <v>13</v>
+      </c>
+      <c r="U59" s="1">
+        <v>21944</v>
+      </c>
+      <c r="V59" s="1">
+        <v>32243</v>
+      </c>
+      <c r="W59" s="1">
+        <v>9416</v>
+      </c>
+      <c r="X59" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y59" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z59" s="1">
+        <v>11.14</v>
+      </c>
+      <c r="AA59" s="1">
+        <v>12.36</v>
+      </c>
+      <c r="AB59" s="1">
+        <v>48.04</v>
+      </c>
+      <c r="AC59" s="1">
+        <v>153.25</v>
+      </c>
+      <c r="AD59" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="AE59" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="60" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.6">
+      <c r="A60" s="1">
+        <v>48</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E60" s="1">
+        <v>4</v>
+      </c>
+      <c r="F60" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="G60" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="H60" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="I60" s="1">
+        <f t="shared" si="10"/>
+        <v>30</v>
+      </c>
+      <c r="J60" s="1">
+        <f t="shared" si="11"/>
+        <v>10</v>
+      </c>
+      <c r="K60" s="1">
+        <v>150000</v>
+      </c>
+      <c r="L60" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="M60" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="N60" s="1">
+        <v>1</v>
+      </c>
+      <c r="O60" s="1">
+        <v>30</v>
+      </c>
+      <c r="P60" s="23"/>
+      <c r="R60" s="1">
+        <v>0.102284</v>
+      </c>
+      <c r="S60" s="1">
+        <v>0.60430200000000001</v>
+      </c>
+      <c r="T60" s="1">
+        <v>9</v>
+      </c>
+      <c r="U60" s="1">
+        <v>432601</v>
+      </c>
+      <c r="V60" s="1">
+        <v>708749</v>
+      </c>
+      <c r="W60" s="1">
+        <v>119440</v>
+      </c>
+      <c r="X60" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y60" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z60" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="AA60" s="1">
+        <v>8.57</v>
+      </c>
+      <c r="AB60" s="1">
+        <v>18.14</v>
+      </c>
+      <c r="AC60" s="1">
+        <v>53.08</v>
+      </c>
+      <c r="AD60" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AE60" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="61" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.6">
+      <c r="A61" s="1">
+        <v>49</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E61" s="1">
+        <v>6</v>
+      </c>
+      <c r="F61" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="G61" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="H61" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="I61" s="1">
+        <f t="shared" si="10"/>
+        <v>100</v>
+      </c>
+      <c r="J61" s="1">
+        <f t="shared" si="11"/>
+        <v>10</v>
+      </c>
+      <c r="K61" s="1">
+        <v>150000</v>
+      </c>
+      <c r="L61" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="M61" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="N61" s="1">
+        <v>1</v>
+      </c>
+      <c r="O61" s="1">
+        <v>100</v>
+      </c>
+      <c r="P61" s="23"/>
+      <c r="R61" s="1">
+        <v>1.7316999999999999E-2</v>
+      </c>
+      <c r="S61" s="1">
+        <v>9.8462999999999995E-2</v>
+      </c>
+      <c r="T61" s="1">
+        <v>9</v>
+      </c>
+      <c r="U61" s="1">
+        <v>432599</v>
+      </c>
+      <c r="V61" s="1">
+        <v>708749</v>
+      </c>
+      <c r="W61" s="1">
+        <v>119440</v>
+      </c>
+      <c r="X61" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y61" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z61" s="1">
+        <v>5.65</v>
+      </c>
+      <c r="AA61" s="1">
+        <v>76.17</v>
+      </c>
+      <c r="AB61" s="1">
+        <v>170.84</v>
+      </c>
+      <c r="AC61" s="1">
+        <v>277.10000000000002</v>
+      </c>
+      <c r="AD61" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="AE61" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="62" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.6">
+      <c r="A62" s="1">
+        <v>51</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E62" s="1">
+        <v>8</v>
+      </c>
+      <c r="F62" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="G62" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="H62" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="I62" s="1">
+        <f>N62*O62</f>
+        <v>400</v>
+      </c>
+      <c r="J62" s="1">
+        <f>G62/F62</f>
+        <v>10</v>
+      </c>
+      <c r="K62" s="1">
+        <v>150000</v>
+      </c>
+      <c r="L62" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="M62" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="N62" s="1">
+        <v>1</v>
+      </c>
+      <c r="O62" s="1">
+        <v>400</v>
+      </c>
+      <c r="P62" s="23"/>
+      <c r="R62" s="1">
+        <v>5.7592999999999998E-2</v>
+      </c>
+      <c r="S62" s="1">
+        <v>0.327463</v>
+      </c>
+      <c r="T62" s="1">
+        <v>9</v>
+      </c>
+      <c r="U62" s="1">
+        <v>432576</v>
+      </c>
+      <c r="V62" s="1">
+        <v>708725</v>
+      </c>
+      <c r="W62" s="1">
+        <v>119440</v>
+      </c>
+      <c r="X62" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y62" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z62" s="1">
+        <v>84.43</v>
+      </c>
+      <c r="AA62" s="1">
+        <v>1070.54</v>
+      </c>
+      <c r="AB62" s="1">
+        <v>2218.6799999999998</v>
+      </c>
+      <c r="AC62" s="1">
+        <v>3401.12</v>
+      </c>
+      <c r="AD62" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="AE62" s="1" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -5846,25 +6447,25 @@
         <v>14</v>
       </c>
       <c r="M1" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="N1" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="O1" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="P1" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="Q1" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="R1" t="s">
         <v>28</v>
       </c>
       <c r="S1" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="T1" t="s">
         <v>30</v>
@@ -5926,10 +6527,10 @@
         <v>124.8</v>
       </c>
       <c r="S2" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T2" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.6">
@@ -5988,10 +6589,10 @@
         <v>125.6</v>
       </c>
       <c r="S3" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T3" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.6">
@@ -6050,10 +6651,10 @@
         <v>126</v>
       </c>
       <c r="S4" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T4" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.6">
@@ -6112,10 +6713,10 @@
         <v>126.8</v>
       </c>
       <c r="S5" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T5" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.6">
@@ -6174,10 +6775,10 @@
         <v>126.9</v>
       </c>
       <c r="S6" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T6" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.6">
@@ -6236,10 +6837,10 @@
         <v>125.7</v>
       </c>
       <c r="S7" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T7" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.6">
@@ -6298,10 +6899,10 @@
         <v>126.9</v>
       </c>
       <c r="S8" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T8" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.6">
@@ -6360,10 +6961,10 @@
         <v>126.6</v>
       </c>
       <c r="S9" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T9" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.6">
@@ -6422,10 +7023,10 @@
         <v>127</v>
       </c>
       <c r="S10" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T10" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.6">
@@ -6484,10 +7085,10 @@
         <v>126.9</v>
       </c>
       <c r="S11" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T11" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.6">
@@ -6546,10 +7147,10 @@
         <v>125.9</v>
       </c>
       <c r="S12" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T12" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.6">
@@ -6608,10 +7209,10 @@
         <v>125.4</v>
       </c>
       <c r="S13" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T13" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.6">
@@ -6670,10 +7271,10 @@
         <v>46.7</v>
       </c>
       <c r="S14" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T14" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.6">
@@ -6732,10 +7333,10 @@
         <v>46.6</v>
       </c>
       <c r="S15" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T15" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.6">
@@ -6794,10 +7395,10 @@
         <v>46.5</v>
       </c>
       <c r="S16" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T16" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.6">
@@ -6856,10 +7457,10 @@
         <v>46.8</v>
       </c>
       <c r="S17" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T17" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.6">
@@ -6918,10 +7519,10 @@
         <v>47.2</v>
       </c>
       <c r="S18" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T18" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.6">
@@ -6980,10 +7581,10 @@
         <v>129.4</v>
       </c>
       <c r="S19" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T19" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.6">
@@ -7042,10 +7643,10 @@
         <v>130.80000000000001</v>
       </c>
       <c r="S20" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T20" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.6">
@@ -7104,10 +7705,10 @@
         <v>129</v>
       </c>
       <c r="S21" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T21" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.6">
@@ -7166,10 +7767,10 @@
         <v>127.9</v>
       </c>
       <c r="S22" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T22" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.6">
@@ -7228,10 +7829,10 @@
         <v>130</v>
       </c>
       <c r="S23" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T23" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.6">
@@ -7290,10 +7891,10 @@
         <v>126.1</v>
       </c>
       <c r="S24" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T24" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.6">
@@ -7352,10 +7953,10 @@
         <v>126.6</v>
       </c>
       <c r="S25" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T25" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.6">
@@ -7414,10 +8015,10 @@
         <v>126</v>
       </c>
       <c r="S26" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T26" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.6">
@@ -7476,10 +8077,10 @@
         <v>125.7</v>
       </c>
       <c r="S27" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T27" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.6">
@@ -7538,10 +8139,10 @@
         <v>127.1</v>
       </c>
       <c r="S28" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T28" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.6">
@@ -7600,10 +8201,10 @@
         <v>126.2</v>
       </c>
       <c r="S29" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T29" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.6">
@@ -7662,10 +8263,10 @@
         <v>125.5</v>
       </c>
       <c r="S30" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T30" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.6">
@@ -7724,10 +8325,10 @@
         <v>127</v>
       </c>
       <c r="S31" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T31" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.6">
@@ -7786,10 +8387,10 @@
         <v>127</v>
       </c>
       <c r="S32" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T32" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.6">
@@ -7848,10 +8449,10 @@
         <v>126.6</v>
       </c>
       <c r="S33" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T33" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.6">
@@ -7910,10 +8511,10 @@
         <v>126.9</v>
       </c>
       <c r="S34" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T34" t="s">
-        <v>185</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.6">
@@ -7972,10 +8573,10 @@
         <v>126.1</v>
       </c>
       <c r="S35" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T35" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.6">
@@ -8034,10 +8635,10 @@
         <v>46.9</v>
       </c>
       <c r="S36" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T36" t="s">
-        <v>187</v>
+        <v>201</v>
       </c>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.6">
@@ -8096,10 +8697,10 @@
         <v>46.7</v>
       </c>
       <c r="S37" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T37" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.6">
@@ -8158,10 +8759,10 @@
         <v>46.9</v>
       </c>
       <c r="S38" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="T38" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.6">
@@ -8220,10 +8821,10 @@
         <v>47</v>
       </c>
       <c r="S39" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="T39" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.6">
@@ -8282,10 +8883,10 @@
         <v>46.6</v>
       </c>
       <c r="S40" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T40" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.6">
@@ -8344,10 +8945,10 @@
         <v>129.6</v>
       </c>
       <c r="S41" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T41" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.6">
@@ -8406,10 +9007,10 @@
         <v>126.3</v>
       </c>
       <c r="S42" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T42" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.6">
@@ -8468,10 +9069,10 @@
         <v>129.9</v>
       </c>
       <c r="S43" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T43" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.6">
@@ -8530,10 +9131,10 @@
         <v>128.5</v>
       </c>
       <c r="S44" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T44" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.6">
@@ -8592,10 +9193,10 @@
         <v>128.30000000000001</v>
       </c>
       <c r="S45" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T45" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.6">
@@ -8654,10 +9255,10 @@
         <v>125.6</v>
       </c>
       <c r="S46" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T46" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.6">
@@ -8716,10 +9317,10 @@
         <v>127.3</v>
       </c>
       <c r="S47" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T47" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.6">
@@ -8778,10 +9379,10 @@
         <v>126.9</v>
       </c>
       <c r="S48" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T48" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.6">
@@ -8840,10 +9441,10 @@
         <v>126.3</v>
       </c>
       <c r="S49" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T49" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.6">
@@ -8902,10 +9503,10 @@
         <v>126.8</v>
       </c>
       <c r="S50" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T50" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
     </row>
     <row r="51" spans="1:20" x14ac:dyDescent="0.6">
@@ -8964,10 +9565,10 @@
         <v>126</v>
       </c>
       <c r="S51" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T51" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.6">
@@ -9026,10 +9627,10 @@
         <v>126.5</v>
       </c>
       <c r="S52" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T52" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
     </row>
     <row r="53" spans="1:20" x14ac:dyDescent="0.6">
@@ -9088,10 +9689,10 @@
         <v>126.8</v>
       </c>
       <c r="S53" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T53" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.6">
@@ -9150,10 +9751,10 @@
         <v>124.4</v>
       </c>
       <c r="S54" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T54" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.6">
@@ -9212,10 +9813,10 @@
         <v>126.5</v>
       </c>
       <c r="S55" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T55" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.6">
@@ -9274,10 +9875,10 @@
         <v>127.1</v>
       </c>
       <c r="S56" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T56" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.6">
@@ -9336,10 +9937,10 @@
         <v>126.7</v>
       </c>
       <c r="S57" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T57" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
     </row>
     <row r="58" spans="1:20" x14ac:dyDescent="0.6">
@@ -9398,10 +9999,10 @@
         <v>46.8</v>
       </c>
       <c r="S58" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T58" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.6">
@@ -9460,10 +10061,10 @@
         <v>46.7</v>
       </c>
       <c r="S59" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="T59" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.6">
@@ -9522,10 +10123,10 @@
         <v>46</v>
       </c>
       <c r="S60" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="T60" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
     </row>
     <row r="61" spans="1:20" x14ac:dyDescent="0.6">
@@ -9584,10 +10185,10 @@
         <v>46.7</v>
       </c>
       <c r="S61" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="T61" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
     </row>
     <row r="62" spans="1:20" x14ac:dyDescent="0.6">
@@ -9646,10 +10247,10 @@
         <v>46.6</v>
       </c>
       <c r="S62" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T62" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.6">
@@ -9708,10 +10309,10 @@
         <v>127.2</v>
       </c>
       <c r="S63" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T63" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.6">
@@ -9770,10 +10371,10 @@
         <v>126.7</v>
       </c>
       <c r="S64" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T64" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.6">
@@ -9832,10 +10433,10 @@
         <v>129.6</v>
       </c>
       <c r="S65" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T65" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.6">
@@ -9894,10 +10495,10 @@
         <v>127.9</v>
       </c>
       <c r="S66" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T66" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.6">
@@ -9956,10 +10557,10 @@
         <v>128</v>
       </c>
       <c r="S67" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="T67" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>